<commit_message>
fix: standardize medical English generic names segmentation across all 738 drugs
</commit_message>
<xml_diff>
--- a/衛生福利部嘉義醫院藥品臨床處方集_115年第二季總表.xlsx
+++ b/衛生福利部嘉義醫院藥品臨床處方集_115年第二季總表.xlsx
@@ -612,7 +612,7 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>MupirocinOint.</t>
+          <t>Mupirocin</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Potassium chloride</t>
+          <t>Potassium Chloride</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride</t>
+          <t>Sodium Chloride 0.45%</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Dextrose</t>
+          <t>Dextrose 10%</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride</t>
+          <t>Sodium Chloride 3%</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>VitaminA/Ergocalciferol/dl-α-Tocophenyl (acetate) Cream</t>
+          <t>Vitamin A / Ergocalciferol (Vit. D2) / dl-α-Tocopherol Acetate (Vit. E)</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>AripiprazoleOralDispersible</t>
+          <t>Aripiprazole</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Aripiprazole (monohydrate)</t>
+          <t>Aripiprazole (Monohydrate)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Derpteextract (Dermatophagoidespteronyssinus),Derfarextract (Dermatophagoidesfarinae)</t>
+          <t>Der p extract (Dermatophagoides pteronyssinus) / Der f extract (Dermatophagoides farinae)</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Propacetamol (HCl)</t>
+          <t>Propacetamol HCl</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1747,7 +1747,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Zoledronic acid</t>
+          <t>Zoledronic Acid</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Acyclovir Cream</t>
+          <t>Acyclovir</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1938,7 +1938,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Acetylcysteine Effervescent</t>
+          <t>Acetylcysteine</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Acetylcysteine Granules</t>
+          <t>Acetylcysteine</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>TPA (RecombinantHumanTissue-TypePlasminogenActivator)</t>
+          <t>Alteplase (Recombinant Human Tissue-Type Plasminogen Activator / t-PA)</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Adapalene Gel</t>
+          <t>Adapalene</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>Benzoylperoxide Gel</t>
+          <t>Benzoyl Peroxide</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Amiodarone (HCl)</t>
+          <t>Amiodarone HCl</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>Chromic chloride hexahydrate/Copper chloride dihydrate/Ferric chloride hexahydrate/Manganese chloride tetrahydrate/Potassium iodide/Sodium fluoride/Sodiummolybdate dihydrate/Zinc chloride/Sodiumselenite anhydrous</t>
+          <t>Chromic Chloride Hexahydrate / Copper Chloride Dihydrate / Ferric Chloride Hexahydrate / Manganese Chloride Tetrahydrate / Potassium Iodide / Sodium Fluoride / Sodium Molybdate Dihydrate / Zinc Chloride / Sodium Selenite Anhydrous</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -2628,7 +2628,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Epinephrine (HCl)</t>
+          <t>Epinephrine HCl</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -2713,7 +2713,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>TetanusToxoid</t>
+          <t>Tetanus Toxoid</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>Biperiden (HCl)</t>
+          <t>Biperiden HCl</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
@@ -2887,7 +2887,7 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Human Albumin</t>
+          <t>Human Serum Albumin 20%</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Aluminumhydroxidedried gel/Magnesiumcarbonatelight/Alginic acid</t>
+          <t>Aluminum Hydroxide Dried Gel / Magnesium Carbonate Light / Alginic Acid</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Thiamine (Vit.B1)/Riboflavin (Vit.B2)</t>
+          <t>Thiamine (Vit. B1) / Riboflavin (Vit. B2)</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>Aluminumdihydroxyallantoinate (=Aldioxa)</t>
+          <t>Aluminum Dihydroxyallantoinate (= Aldioxa)</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Palonosetron (HCl)</t>
+          <t>Palonosetron HCl</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Aluminumhydroxide gel</t>
+          <t>Aluminum Hydroxide Gel</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>CiclesonideInhaler</t>
+          <t>Ciclesonide</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr">
@@ -3885,7 +3885,7 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Glimepiride/Metformin (HCl)</t>
+          <t>Glimepiride / Metformin HCl</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="G41" s="3" t="inlineStr">
         <is>
-          <t>Ambroxol (HCl)</t>
+          <t>Ambroxol HCl</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Ampicillin (sodium)/Sulbactam (sodium)</t>
+          <t>Ampicillin Sodium / Sulbactam Sodium</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Amlodipine (besylate)/Benazepril (HCl)</t>
+          <t>Amlodipine Besylate / Benazepril HCl</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="G49" s="3" t="inlineStr">
         <is>
-          <t>Acetaminophen/Orphenadrine citrate</t>
+          <t>Acetaminophen / Orphenadrine Citrate</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>Amoxicillin (sodium)/Clavulanic acid (potassium)</t>
+          <t>Amoxicillin Sodium / Clavulanate Potassium</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Umeclidinium bromide/VilanteroltrifenatateInh.Powder</t>
+          <t>Umeclidinium Bromide / Vilanterol Trifenatate</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr">
@@ -5128,7 +5128,7 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>LactobacillusCaseiVarietyRhamnosus</t>
+          <t>Lactobacillus Casei Variety Rhamnosus</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>ChlorhexidinegluconateSol'n</t>
+          <t>Chlorhexidine Gluconate</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr">
@@ -5553,7 +5553,7 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>MirtazapineOralDispersible</t>
+          <t>Mirtazapine</t>
         </is>
       </c>
       <c r="H58" s="3" t="inlineStr">
@@ -5731,7 +5731,7 @@
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Valproic acid (=Valproate)</t>
+          <t>Valproic Acid (=Valproate)</t>
         </is>
       </c>
       <c r="H60" s="3" t="inlineStr">
@@ -5816,7 +5816,7 @@
       </c>
       <c r="G61" s="3" t="inlineStr">
         <is>
-          <t>Valproic acid (=Valproate)</t>
+          <t>Valproic Acid (=Valproate)</t>
         </is>
       </c>
       <c r="H61" s="3" t="inlineStr">
@@ -6615,7 +6615,7 @@
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>HydroxypropylmethylcelluloseOph.Sol'n</t>
+          <t>Hydroxypropyl Methylcellulose (Hypromellose)</t>
         </is>
       </c>
       <c r="H70" s="3" t="inlineStr">
@@ -6704,7 +6704,7 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>MesalazineSupp.</t>
+          <t>Mesalazine</t>
         </is>
       </c>
       <c r="H71" s="3" t="inlineStr">
@@ -7032,7 +7032,7 @@
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>SodiumchlorideEnema</t>
+          <t>Sodium Chloride</t>
         </is>
       </c>
       <c r="H75" s="3" t="inlineStr">
@@ -7201,7 +7201,7 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>AzelastineHClNasal Spray</t>
+          <t>Azelastine HCl</t>
         </is>
       </c>
       <c r="H77" s="3" t="inlineStr">
@@ -7371,7 +7371,7 @@
       </c>
       <c r="G79" s="3" t="inlineStr">
         <is>
-          <t>Benzylbenzoate Lotion</t>
+          <t>Benzyl Benzoate</t>
         </is>
       </c>
       <c r="H79" s="3" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>Sulfamethoxazole/Trimethoprim</t>
+          <t>Sulfamethoxazole / Trimethoprim</t>
         </is>
       </c>
       <c r="H80" s="3" t="inlineStr">
@@ -7547,7 +7547,7 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>Pyridoxine (Vit.B6)(HCl)</t>
+          <t>Pyridoxine (Vit. B6)(HCl)</t>
         </is>
       </c>
       <c r="H81" s="3" t="inlineStr">
@@ -7802,7 +7802,7 @@
       </c>
       <c r="G84" s="3" t="inlineStr">
         <is>
-          <t>IpratropiumBr/SalbutamolInhaler</t>
+          <t>Ipratropium Bromide / Salbutamol</t>
         </is>
       </c>
       <c r="H84" s="3" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="G85" s="3" t="inlineStr">
         <is>
-          <t>Clobetasolpropionate Cream</t>
+          <t>Clobetasol Propionate</t>
         </is>
       </c>
       <c r="H85" s="3" t="inlineStr">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="G86" s="3" t="inlineStr">
         <is>
-          <t>Piperacillin (sodium)/Tazobactam (sodium)</t>
+          <t>Piperacillin Sodium / Tazobactam Sodium</t>
         </is>
       </c>
       <c r="H86" s="3" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="G89" s="3" t="inlineStr">
         <is>
-          <t>L-Leucine/L-Isoleucine/L-Valine/L-Lysine (HCl)/L-Threonine/L-Tryptophan/Acetylcysteine/L-Phenylalanine/L-Arginine/L-Alanine/L-Serine/L-Aspartic acid/Dibasicpotassium phosphate/Sodiumcitrate Hydrate/L-Methionine/L-Tyrosine/L-Histidine/L-Proline/Glycine/L-Glutamic acid/Dibasicsodiumphosphate Hydrate/SodiumlactateSol'n/Glucose/Calciumchloride hydrate/Zincsulfate hydrate/Potassium chloride/Magnesiumsulfate hydrate/Thiamine (Vit.B1)(HCl)</t>
+          <t>Amino Acids / Glucose / Electrolytes (BCAA 30% / Thiamine)</t>
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
@@ -8330,7 +8330,7 @@
       </c>
       <c r="G90" s="3" t="inlineStr">
         <is>
-          <t>Tenofoviralafenamide/Emtricitabine/Bictegravir</t>
+          <t>Bictegravir / Emtricitabine / Tenofovir Alafenamide</t>
         </is>
       </c>
       <c r="H90" s="3" t="inlineStr">
@@ -8694,7 +8694,7 @@
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t>Povidone-IodineOint.</t>
+          <t>Povidone-Iodine</t>
         </is>
       </c>
       <c r="H94" s="3" t="inlineStr">
@@ -8783,7 +8783,7 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t>Neomycin (Fradiomycin)(sulfate)/TyrothricinOint.</t>
+          <t>Neomycin (Fradiomycin) Sulfate / Tyrothricin</t>
         </is>
       </c>
       <c r="H95" s="3" t="inlineStr">
@@ -8868,7 +8868,7 @@
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>BisacodylSupp.</t>
+          <t>Bisacodyl</t>
         </is>
       </c>
       <c r="H96" s="3" t="inlineStr">
@@ -9042,7 +9042,7 @@
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>Bisoprolol fumarate (=hemifumarate)</t>
+          <t>Bisoprololfumarate (=hemifumarate)</t>
         </is>
       </c>
       <c r="H98" s="3" t="inlineStr">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t>Candesartancilexetil</t>
+          <t>Candesartan Cilexetil</t>
         </is>
       </c>
       <c r="H100" s="3" t="inlineStr">
@@ -9297,7 +9297,7 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t>Calciumphosphatetribasic/VitaminA/VitaminA (VitaminA+VitaminD) Emulsion</t>
+          <t>Calcium Phosphate Tribasic / Vitamin A / Vitamin D</t>
         </is>
       </c>
       <c r="H101" s="3" t="inlineStr">
@@ -9382,7 +9382,7 @@
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>Ibandronic acid</t>
+          <t>Ibandronic Acid</t>
         </is>
       </c>
       <c r="H102" s="3" t="inlineStr">
@@ -9471,7 +9471,7 @@
       </c>
       <c r="G103" s="3" t="inlineStr">
         <is>
-          <t>Picosulfate sodium/Citric acid anhydrous/Magnesium oxide</t>
+          <t>Sodium Picosulfate / Citric Acid Anhydrous / Magnesium Oxide</t>
         </is>
       </c>
       <c r="H103" s="3" t="inlineStr">
@@ -9554,7 +9554,7 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t>Sugammadex</t>
+          <t>Sugammadex Sodium</t>
         </is>
       </c>
       <c r="H104" s="3" t="inlineStr">
@@ -9817,7 +9817,7 @@
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t>Cefoperazone (sodium)/Sulbactam (sodium)</t>
+          <t>Cefoperazone Sodium / Sulbactam Sodium</t>
         </is>
       </c>
       <c r="H107" s="3" t="inlineStr">
@@ -10003,7 +10003,7 @@
       </c>
       <c r="G109" s="3" t="inlineStr">
         <is>
-          <t>Cefoperazone /Sulbactam</t>
+          <t>Cefoperazone Sodium / Sulbactam Sodium</t>
         </is>
       </c>
       <c r="H109" s="3" t="inlineStr">
@@ -10072,7 +10072,7 @@
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>Hyoscine (Scopolamine)-N-Butyl bromide</t>
+          <t>Hyoscine (Scopolamine)-N-Butylbromide</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr">
@@ -10246,7 +10246,7 @@
       </c>
       <c r="G112" s="3" t="inlineStr">
         <is>
-          <t>Terbutaline (sulfate) Inh.Sol'n</t>
+          <t>Terbutaline (sulfate) Inh.</t>
         </is>
       </c>
       <c r="H112" s="3" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="G113" s="3" t="inlineStr">
         <is>
-          <t>Remimazolam besylate</t>
+          <t>Remimazolambesylate</t>
         </is>
       </c>
       <c r="H113" s="3" t="inlineStr">
@@ -10420,7 +10420,7 @@
       </c>
       <c r="G114" s="3" t="inlineStr">
         <is>
-          <t>Chlorpheniramine (maleate)/Lidocaine (HCl)/Camphor/Menthol/MethylsalicylateOint.</t>
+          <t>Chlorpheniramine Maleate / Lidocaine HCl / Methyl Salicylate / Menthol / Camphor</t>
         </is>
       </c>
       <c r="H114" s="3" t="inlineStr">
@@ -10597,7 +10597,7 @@
       </c>
       <c r="G116" s="3" t="inlineStr">
         <is>
-          <t>Amlodipine (besylate)/Atorvastatin (calcium)</t>
+          <t>Amlodipine Besylate / Atorvastatin Calcium</t>
         </is>
       </c>
       <c r="H116" s="3" t="inlineStr">
@@ -10682,7 +10682,7 @@
       </c>
       <c r="G117" s="3" t="inlineStr">
         <is>
-          <t>Calcium carbonate</t>
+          <t>Calciumcarbonate</t>
         </is>
       </c>
       <c r="H117" s="3" t="inlineStr">
@@ -10771,7 +10771,7 @@
       </c>
       <c r="G118" s="3" t="inlineStr">
         <is>
-          <t>Calciumphosphatedibasic/Calcium gluconate/Ergocalciferol (Vit.D2)</t>
+          <t>Calcium Phosphate Dibasic / Calcium Gluconate / Ergocalciferol (Vit. D2)</t>
         </is>
       </c>
       <c r="H118" s="3" t="inlineStr">
@@ -10860,7 +10860,7 @@
       </c>
       <c r="G119" s="3" t="inlineStr">
         <is>
-          <t>CalcipotriolOint.</t>
+          <t>Calcipotriol</t>
         </is>
       </c>
       <c r="H119" s="3" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="G122" s="3" t="inlineStr">
         <is>
-          <t>Sulfadiazinesilver Cream</t>
+          <t>Silver Sulfadiazine</t>
         </is>
       </c>
       <c r="H122" s="3" t="inlineStr">
@@ -11206,7 +11206,7 @@
       </c>
       <c r="G123" s="3" t="inlineStr">
         <is>
-          <t>Activatedcharcoal Granules</t>
+          <t>Activated Charcoal</t>
         </is>
       </c>
       <c r="H123" s="3" t="inlineStr">
@@ -11465,7 +11465,7 @@
       </c>
       <c r="G126" s="3" t="inlineStr">
         <is>
-          <t>Carisoprodol/Acetaminophen/Caffeine</t>
+          <t>Carisoprodol / Acetaminophen / Caffeine</t>
         </is>
       </c>
       <c r="H126" s="3" t="inlineStr">
@@ -11886,7 +11886,7 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Nicotinamine (Vit.B3)/Thiamine (Vit.B1)/Riboflavin (Vit.B2) phosphate/Pyridoxine (Vit.B6)/Ascorbic acid</t>
+          <t>Nicotinamide (Vit. B3) / Thiamine (Vit. B1) / Riboflavin (Vit. B2) / Pyridoxine (Vit. B6) / Ascorbic Acid (Vit. C)</t>
         </is>
       </c>
       <c r="H131" s="3" t="inlineStr">
@@ -12330,7 +12330,7 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t>Cetirizine (2HCl) OralSol'n</t>
+          <t>Cetirizine 2HCl</t>
         </is>
       </c>
       <c r="H136" s="3" t="inlineStr">
@@ -12500,7 +12500,7 @@
       </c>
       <c r="G138" s="3" t="inlineStr">
         <is>
-          <t>Varenicline (tartrate)</t>
+          <t>Varenicline Tartrate</t>
         </is>
       </c>
       <c r="H138" s="3" t="inlineStr">
@@ -12589,7 +12589,7 @@
       </c>
       <c r="G139" s="3" t="inlineStr">
         <is>
-          <t>DesoximetasoneOint.</t>
+          <t>Desoximetasone</t>
         </is>
       </c>
       <c r="H139" s="3" t="inlineStr">
@@ -12845,7 +12845,7 @@
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>Heparinoid Gel</t>
+          <t>Heparinoid</t>
         </is>
       </c>
       <c r="H142" s="3" t="inlineStr">
@@ -12936,7 +12936,7 @@
       </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
-          <t>EthanolSol'n</t>
+          <t>Ethanol 75%</t>
         </is>
       </c>
       <c r="H143" s="3" t="inlineStr">
@@ -13376,7 +13376,7 @@
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t>Valsartan/Hydrochlorothiazide</t>
+          <t>Valsartan / Hydrochlorothiazide</t>
         </is>
       </c>
       <c r="H148" s="3" t="inlineStr">
@@ -13466,7 +13466,7 @@
       </c>
       <c r="G149" s="3" t="inlineStr">
         <is>
-          <t>Colchicine</t>
+          <t>Polyethylene Glycol 3350 / Sodium Sulfate Anhydrous / Sodium Bicarbonate / Sodium Chloride / Potassium Chloride</t>
         </is>
       </c>
       <c r="H149" s="3" t="inlineStr">
@@ -13551,7 +13551,7 @@
       </c>
       <c r="G150" s="3" t="inlineStr">
         <is>
-          <t>Colistimethate sodium (SterilesodiumColistin methanesulfonate)</t>
+          <t>Colistimethate Sodium (Sterile Sodium Colistin)</t>
         </is>
       </c>
       <c r="H150" s="3" t="inlineStr">
@@ -13640,7 +13640,7 @@
       </c>
       <c r="G151" s="3" t="inlineStr">
         <is>
-          <t>Bisoprolol fumarate (=hemifumarate)</t>
+          <t>Bisoprololfumarate (=hemifumarate)</t>
         </is>
       </c>
       <c r="H151" s="3" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="G152" s="3" t="inlineStr">
         <is>
-          <t>Potassium chloride</t>
+          <t>Potassium Chloride</t>
         </is>
       </c>
       <c r="H152" s="3" t="inlineStr">
@@ -13812,7 +13812,7 @@
       </c>
       <c r="G153" s="3" t="inlineStr">
         <is>
-          <t>Bupropion/Naltrexone</t>
+          <t>Bupropion HCl / Naltrexone HCl</t>
         </is>
       </c>
       <c r="H153" s="3" t="inlineStr">
@@ -14150,7 +14150,7 @@
       </c>
       <c r="G157" s="3" t="inlineStr">
         <is>
-          <t>Estradiol/Norethindrone (acetate)</t>
+          <t>Estradiol / Norethindrone Acetate</t>
         </is>
       </c>
       <c r="H157" s="3" t="inlineStr">
@@ -14410,7 +14410,7 @@
       </c>
       <c r="G160" s="3" t="inlineStr">
         <is>
-          <t>Levofloxacin hemihydrate</t>
+          <t>Levofloxacinhemihydrate</t>
         </is>
       </c>
       <c r="H160" s="3" t="inlineStr">
@@ -14499,7 +14499,7 @@
       </c>
       <c r="G161" s="3" t="inlineStr">
         <is>
-          <t>Levofloxacin hemihydrate</t>
+          <t>Levofloxacinhemihydrate</t>
         </is>
       </c>
       <c r="H161" s="3" t="inlineStr">
@@ -14588,7 +14588,7 @@
       </c>
       <c r="G162" s="3" t="inlineStr">
         <is>
-          <t>LevofloxacinOph.Sol'n</t>
+          <t>Levofloxacin</t>
         </is>
       </c>
       <c r="H162" s="3" t="inlineStr">
@@ -14855,7 +14855,7 @@
       </c>
       <c r="G165" s="3" t="inlineStr">
         <is>
-          <t>Amoxicillin (trihydrate)/Clavulanic acid</t>
+          <t>Amoxicillin Trihydrate / Clavulanic Acid</t>
         </is>
       </c>
       <c r="H165" s="3" t="inlineStr">
@@ -14944,7 +14944,7 @@
       </c>
       <c r="G166" s="3" t="inlineStr">
         <is>
-          <t>Amoxicillin (trihydrate)/ClavulanatePowderforOralSusp.</t>
+          <t>Amoxicillin Trihydrate / Clavulanate Potassium</t>
         </is>
       </c>
       <c r="H166" s="3" t="inlineStr">
@@ -15118,7 +15118,7 @@
       </c>
       <c r="G168" s="3" t="inlineStr">
         <is>
-          <t>Betamethasone dipropionate/CalcipotriolOint.</t>
+          <t>Betamethasone Dipropionate / Calcipotriol</t>
         </is>
       </c>
       <c r="H168" s="3" t="inlineStr">
@@ -15210,7 +15210,7 @@
       </c>
       <c r="G169" s="3" t="inlineStr">
         <is>
-          <t>Solifenacin succinate</t>
+          <t>Solifenacinsuccinate</t>
         </is>
       </c>
       <c r="H169" s="3" t="inlineStr">
@@ -15993,7 +15993,7 @@
       </c>
       <c r="G178" s="3" t="inlineStr">
         <is>
-          <t>Dexamethasone (sodium phosphate)/Neomycin (Fradiomycin) Oph.Sol'n</t>
+          <t>Dexamethasone Sodium Phosphate / Neomycin (Fradiomycin) Sulfate</t>
         </is>
       </c>
       <c r="H178" s="3" t="inlineStr">
@@ -16082,7 +16082,7 @@
       </c>
       <c r="G179" s="3" t="inlineStr">
         <is>
-          <t>Doravirine/Lamivudine/Tenofovirdisoproxil fumarate</t>
+          <t>Doravirine / Lamivudine / Tenofovir Disoproxil Fumarate</t>
         </is>
       </c>
       <c r="H179" s="3" t="inlineStr">
@@ -16309,7 +16309,7 @@
       </c>
       <c r="G182" s="3" t="inlineStr">
         <is>
-          <t>Valproic acid (=Valproate)</t>
+          <t>Valproic Acid (=Valproate)</t>
         </is>
       </c>
       <c r="H182" s="3" t="inlineStr">
@@ -16402,7 +16402,7 @@
       </c>
       <c r="G183" s="3" t="inlineStr">
         <is>
-          <t>Dexamethasone (sodium phosphate)</t>
+          <t>Dexamethasone (sodiumphosphate)</t>
         </is>
       </c>
       <c r="H183" s="3" t="inlineStr">
@@ -16487,7 +16487,7 @@
       </c>
       <c r="G184" s="3" t="inlineStr">
         <is>
-          <t>Dextrose/Sodium chloride</t>
+          <t>Dextrose / Sodium Chloride</t>
         </is>
       </c>
       <c r="H184" s="3" t="inlineStr">
@@ -16645,7 +16645,7 @@
       </c>
       <c r="G186" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H186" s="3" t="inlineStr">
@@ -16734,7 +16734,7 @@
       </c>
       <c r="G187" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H187" s="3" t="inlineStr">
@@ -16823,7 +16823,7 @@
       </c>
       <c r="G188" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H188" s="3" t="inlineStr">
@@ -16912,7 +16912,7 @@
       </c>
       <c r="G189" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H189" s="3" t="inlineStr">
@@ -17001,7 +17001,7 @@
       </c>
       <c r="G190" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith2.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 2.5% Dextrose)</t>
         </is>
       </c>
       <c r="H190" s="3" t="inlineStr">
@@ -17090,7 +17090,7 @@
       </c>
       <c r="G191" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith2.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 2.5% Dextrose)</t>
         </is>
       </c>
       <c r="H191" s="3" t="inlineStr">
@@ -17179,7 +17179,7 @@
       </c>
       <c r="G192" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwith2.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 2.5% Dextrose)</t>
         </is>
       </c>
       <c r="H192" s="3" t="inlineStr">
@@ -17268,7 +17268,7 @@
       </c>
       <c r="G193" s="3" t="inlineStr">
         <is>
-          <t>DianealLow Calcium (2.5mEq/L) PeritonealdialysisSol'nwithDextrose4.25%</t>
+          <t>Peritoneal Dialysis Solution (Low Calcium 2.5 mEq/L with 4.25% Dextrose)</t>
         </is>
       </c>
       <c r="H193" s="3" t="inlineStr">
@@ -17357,7 +17357,7 @@
       </c>
       <c r="G194" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H194" s="3" t="inlineStr">
@@ -17446,7 +17446,7 @@
       </c>
       <c r="G195" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H195" s="3" t="inlineStr">
@@ -17535,7 +17535,7 @@
       </c>
       <c r="G196" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H196" s="3" t="inlineStr">
@@ -17624,7 +17624,7 @@
       </c>
       <c r="G197" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealDialysisSol'nwith1.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 1.5% Dextrose)</t>
         </is>
       </c>
       <c r="H197" s="3" t="inlineStr">
@@ -17713,7 +17713,7 @@
       </c>
       <c r="G198" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith2.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 2.5% Dextrose)</t>
         </is>
       </c>
       <c r="H198" s="3" t="inlineStr">
@@ -17802,7 +17802,7 @@
       </c>
       <c r="G199" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith2.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 2.5% Dextrose)</t>
         </is>
       </c>
       <c r="H199" s="3" t="inlineStr">
@@ -17891,7 +17891,7 @@
       </c>
       <c r="G200" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith2.5%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 2.5% Dextrose)</t>
         </is>
       </c>
       <c r="H200" s="3" t="inlineStr">
@@ -17980,7 +17980,7 @@
       </c>
       <c r="G201" s="3" t="inlineStr">
         <is>
-          <t>DianealPD-2PeritonealdialysisSol'nwith4.25%Dextrose</t>
+          <t>Peritoneal Dialysis Solution (PD-2 with 4.25% Dextrose)</t>
         </is>
       </c>
       <c r="H201" s="3" t="inlineStr">
@@ -18235,7 +18235,7 @@
       </c>
       <c r="G204" s="3" t="inlineStr">
         <is>
-          <t>Diclofenac (sodium) Supp.</t>
+          <t>Diclofenac (sodium) .</t>
         </is>
       </c>
       <c r="H204" s="3" t="inlineStr">
@@ -18320,7 +18320,7 @@
       </c>
       <c r="G205" s="3" t="inlineStr">
         <is>
-          <t>Chlorpheniramine (maleate)/Methylephedrinedl-(HCl)/Codeine (phosphate)/PotassiumGuaiacolSulfonate Syrup</t>
+          <t>Chlorpheniramine (maleate) / Methylephedrinedl-(HCl) / Codeine (phosphate) / Potassium Guaiacol Sulfonate Syrup</t>
         </is>
       </c>
       <c r="H205" s="3" t="inlineStr">
@@ -18749,7 +18749,7 @@
       </c>
       <c r="G210" s="3" t="inlineStr">
         <is>
-          <t>FlurbiprofenPatch</t>
+          <t>Flurbiprofen Patch</t>
         </is>
       </c>
       <c r="H210" s="3" t="inlineStr">
@@ -18838,7 +18838,7 @@
       </c>
       <c r="G211" s="3" t="inlineStr">
         <is>
-          <t>Estradiol Gel</t>
+          <t>Estradiol</t>
         </is>
       </c>
       <c r="H211" s="3" t="inlineStr">
@@ -18931,7 +18931,7 @@
       </c>
       <c r="G212" s="3" t="inlineStr">
         <is>
-          <t>Donepezil (HCl) OralDispersible</t>
+          <t>Donepezil (HCl)</t>
         </is>
       </c>
       <c r="H212" s="3" t="inlineStr">
@@ -19190,7 +19190,7 @@
       </c>
       <c r="G215" s="3" t="inlineStr">
         <is>
-          <t>Dota/Gadolinium oxide</t>
+          <t>Dota / Gadoliniumoxide</t>
         </is>
       </c>
       <c r="H215" s="3" t="inlineStr">
@@ -19277,7 +19277,7 @@
       </c>
       <c r="G216" s="3" t="inlineStr">
         <is>
-          <t>Dolutegravir/Lamivudine</t>
+          <t>Dolutegravir / Lamivudine</t>
         </is>
       </c>
       <c r="H216" s="3" t="inlineStr">
@@ -19536,7 +19536,7 @@
       </c>
       <c r="G219" s="3" t="inlineStr">
         <is>
-          <t>AzelastineHCl/FluticasoneNasal Spray</t>
+          <t>Azelastine HCl / Fluticasone</t>
         </is>
       </c>
       <c r="H219" s="3" t="inlineStr">
@@ -20159,7 +20159,7 @@
       </c>
       <c r="G226" s="3" t="inlineStr">
         <is>
-          <t>Policresulen/Cinchocaine (HCl) Supp.</t>
+          <t>Policresulen / Cinchocaine (HCl) .</t>
         </is>
       </c>
       <c r="H226" s="3" t="inlineStr">
@@ -20503,7 +20503,7 @@
       </c>
       <c r="G230" s="3" t="inlineStr">
         <is>
-          <t>Emedastine (difumarate) Oph.Sol'n</t>
+          <t>Emedastine (difumarate) Oph.</t>
         </is>
       </c>
       <c r="H230" s="3" t="inlineStr">
@@ -20680,7 +20680,7 @@
       </c>
       <c r="G232" s="3" t="inlineStr">
         <is>
-          <t>HepatitisB,antigen,surface</t>
+          <t>Hepatitis B / antigen / surface</t>
         </is>
       </c>
       <c r="H232" s="3" t="inlineStr">
@@ -20941,7 +20941,7 @@
       </c>
       <c r="G235" s="3" t="inlineStr">
         <is>
-          <t>Sacubitril/Valsartan (sodium)</t>
+          <t>Sacubitril / Valsartan (sodium)</t>
         </is>
       </c>
       <c r="H235" s="3" t="inlineStr">
@@ -21038,7 +21038,7 @@
       </c>
       <c r="G236" s="3" t="inlineStr">
         <is>
-          <t>Sofosbuvir/Velpatasvir</t>
+          <t>Sofosbuvir / Velpatasvir</t>
         </is>
       </c>
       <c r="H236" s="3" t="inlineStr">
@@ -21208,7 +21208,7 @@
       </c>
       <c r="G238" s="3" t="inlineStr">
         <is>
-          <t>EpinephrineSol'n</t>
+          <t>Epinephrine</t>
         </is>
       </c>
       <c r="H238" s="3" t="inlineStr">
@@ -21382,7 +21382,7 @@
       </c>
       <c r="G240" s="3" t="inlineStr">
         <is>
-          <t>ErythromycinOph.Oint.</t>
+          <t>Erythromycin Oph..</t>
         </is>
       </c>
       <c r="H240" s="3" t="inlineStr">
@@ -21467,7 +21467,7 @@
       </c>
       <c r="G241" s="3" t="inlineStr">
         <is>
-          <t>Acetylsalicylic acid (Aspirin)</t>
+          <t>Acetylsalicylic Acid (Aspirin)</t>
         </is>
       </c>
       <c r="H241" s="3" t="inlineStr">
@@ -21556,7 +21556,7 @@
       </c>
       <c r="G242" s="3" t="inlineStr">
         <is>
-          <t>ConjugatedEstrogen</t>
+          <t>Conjugated Estrogen</t>
         </is>
       </c>
       <c r="H242" s="3" t="inlineStr">
@@ -21819,7 +21819,7 @@
       </c>
       <c r="G245" s="3" t="inlineStr">
         <is>
-          <t>Nicametate citrate</t>
+          <t>Nicametatecitrate</t>
         </is>
       </c>
       <c r="H245" s="3" t="inlineStr">
@@ -22075,7 +22075,7 @@
       </c>
       <c r="G248" s="3" t="inlineStr">
         <is>
-          <t>Sodiumphosphatedibasic anhydrous/SodiumphosphatemonobasicanhydrousEnema</t>
+          <t>Dibasic Sodium Phosphate Anhydrous / Monobasic Sodium Phosphate Anhydrous</t>
         </is>
       </c>
       <c r="H248" s="3" t="inlineStr">
@@ -22351,7 +22351,7 @@
       </c>
       <c r="G251" s="3" t="inlineStr">
         <is>
-          <t>Memantine (HCl)</t>
+          <t>Memantine HCl</t>
         </is>
       </c>
       <c r="H251" s="3" t="inlineStr">
@@ -22438,7 +22438,7 @@
       </c>
       <c r="G252" s="3" t="inlineStr">
         <is>
-          <t>Rivastigminehydrogen tartrate</t>
+          <t>Rivastigminehydrogentartrate</t>
         </is>
       </c>
       <c r="H252" s="3" t="inlineStr">
@@ -22527,7 +22527,7 @@
       </c>
       <c r="G253" s="3" t="inlineStr">
         <is>
-          <t>RivastigminePatch</t>
+          <t>Rivastigmine Patch</t>
         </is>
       </c>
       <c r="H253" s="3" t="inlineStr">
@@ -22616,7 +22616,7 @@
       </c>
       <c r="G254" s="3" t="inlineStr">
         <is>
-          <t>Amlodipine (besylate)/Valsartan</t>
+          <t>Amlodipine (besylate) / Valsartan</t>
         </is>
       </c>
       <c r="H254" s="3" t="inlineStr">
@@ -22705,7 +22705,7 @@
       </c>
       <c r="G255" s="3" t="inlineStr">
         <is>
-          <t>Amlodipine (besylate)/Valsartan/Hydrochlorothiazide</t>
+          <t>Amlodipine (besylate) / Valsartan / Hydrochlorothiazide</t>
         </is>
       </c>
       <c r="H255" s="3" t="inlineStr">
@@ -22875,7 +22875,7 @@
       </c>
       <c r="G257" s="3" t="inlineStr">
         <is>
-          <t>ExtranealPeritonealDialysisSol'nwith7.5%Icodextrin</t>
+          <t>Icodextrin 7.5% (Peritoneal Dialysis Solution)</t>
         </is>
       </c>
       <c r="H257" s="3" t="inlineStr">
@@ -22968,7 +22968,7 @@
       </c>
       <c r="G258" s="3" t="inlineStr">
         <is>
-          <t>ExtranealPeritonealDialysisSol'nwith7.5%Icodextrin</t>
+          <t>Icodextrin 7.5% (Peritoneal Dialysis Solution)</t>
         </is>
       </c>
       <c r="H258" s="3" t="inlineStr">
@@ -23041,7 +23041,7 @@
       </c>
       <c r="G259" s="3" t="inlineStr">
         <is>
-          <t>Betamethasone/Neomycin (Fradiomycin) EyeOint</t>
+          <t>Betamethasone / Neomycin (Fradiomycin) Eye</t>
         </is>
       </c>
       <c r="H259" s="3" t="inlineStr">
@@ -23806,7 +23806,7 @@
       </c>
       <c r="G268" s="3" t="inlineStr">
         <is>
-          <t>FluorometholoneOph.Susp.</t>
+          <t>Fluorometholone Oph..</t>
         </is>
       </c>
       <c r="H268" s="3" t="inlineStr">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="G271" s="3" t="inlineStr">
         <is>
-          <t>Folic acid</t>
+          <t>Folic Acid</t>
         </is>
       </c>
       <c r="H271" s="3" t="inlineStr">
@@ -24312,7 +24312,7 @@
       </c>
       <c r="G274" s="3" t="inlineStr">
         <is>
-          <t>MetronidazoleVag.Supp.</t>
+          <t>Metronidazole Vag..</t>
         </is>
       </c>
       <c r="H274" s="3" t="inlineStr">
@@ -24379,7 +24379,7 @@
       </c>
       <c r="G275" s="3" t="inlineStr">
         <is>
-          <t>Econazole nitrate/Triamcinoloneacetonide Cream</t>
+          <t>Econazolenitrate / Triamcinoloneacetonide</t>
         </is>
       </c>
       <c r="H275" s="3" t="inlineStr">
@@ -24639,7 +24639,7 @@
       </c>
       <c r="G278" s="3" t="inlineStr">
         <is>
-          <t>Fusidic acid Cream</t>
+          <t>Fusidic Acid</t>
         </is>
       </c>
       <c r="H278" s="3" t="inlineStr">
@@ -24898,7 +24898,7 @@
       </c>
       <c r="G281" s="3" t="inlineStr">
         <is>
-          <t>Vildagliptin/Metformin (HCl)</t>
+          <t>Vildagliptin / Metformin (HCl)</t>
         </is>
       </c>
       <c r="H281" s="3" t="inlineStr">
@@ -25080,7 +25080,7 @@
       </c>
       <c r="G283" s="3" t="inlineStr">
         <is>
-          <t>HumanPapillomavirusVaccineType6,11,16,18,31,33,45,52,58</t>
+          <t>Human Papillomavirus Vaccine Type6 / 11 / 16 / 18 / 31 / 33 / 45 / 52 / 58</t>
         </is>
       </c>
       <c r="H283" s="3" t="inlineStr">
@@ -25169,7 +25169,7 @@
       </c>
       <c r="G284" s="3" t="inlineStr">
         <is>
-          <t>Famotidine Granules</t>
+          <t>Famotidine</t>
         </is>
       </c>
       <c r="H284" s="3" t="inlineStr">
@@ -25242,7 +25242,7 @@
       </c>
       <c r="G285" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride/Succinylategelatin</t>
+          <t>Sodium Chloride / Succinylategelatin</t>
         </is>
       </c>
       <c r="H285" s="3" t="inlineStr">
@@ -25594,7 +25594,7 @@
       </c>
       <c r="G289" s="3" t="inlineStr">
         <is>
-          <t>Tenofoviralafenamide/Emtricitabine/Elvitegravir/Cobicistat</t>
+          <t>Tenofovir Alafenamide / Emtricitabine / Elvitegravir / Cobicistat</t>
         </is>
       </c>
       <c r="H289" s="3" t="inlineStr">
@@ -25768,7 +25768,7 @@
       </c>
       <c r="G291" s="3" t="inlineStr">
         <is>
-          <t>Polyethyleneglycol3350/Sodium sulfate anhydrous/Sodium bicarbonate/Sodium chloride/Potassium chloride</t>
+          <t>Polyethyleneglycol3350 / Sodiumsulfateanhydrous / Sodium Bicarbonate / Sodium Chloride / Potassium Chloride</t>
         </is>
       </c>
       <c r="H291" s="3" t="inlineStr">
@@ -25851,7 +25851,7 @@
       </c>
       <c r="G292" s="3" t="inlineStr">
         <is>
-          <t>GinkgoBilobaExtract</t>
+          <t>Ginkgo Biloba Extract</t>
         </is>
       </c>
       <c r="H292" s="3" t="inlineStr">
@@ -26025,7 +26025,7 @@
       </c>
       <c r="G294" s="3" t="inlineStr">
         <is>
-          <t>Dopamine (HCl)/Glucose</t>
+          <t>Dopamine (HCl) / Glucose</t>
         </is>
       </c>
       <c r="H294" s="3" t="inlineStr">
@@ -26289,7 +26289,7 @@
       </c>
       <c r="G297" s="3" t="inlineStr">
         <is>
-          <t>Empagliflozin/Linagliptin</t>
+          <t>Empagliflozin / Linagliptin</t>
         </is>
       </c>
       <c r="H297" s="3" t="inlineStr">
@@ -26382,7 +26382,7 @@
       </c>
       <c r="G298" s="3" t="inlineStr">
         <is>
-          <t>Irontrivalent (Ferric-Hydr oxide-SucroseCompex)</t>
+          <t>Irontrivalent (Ferric-Hydroxide-Sucrose Compex)</t>
         </is>
       </c>
       <c r="H298" s="3" t="inlineStr">
@@ -26467,7 +26467,7 @@
       </c>
       <c r="G299" s="3" t="inlineStr">
         <is>
-          <t>Povidone-IodineAq.Sol'n</t>
+          <t>Povidone-Iodine Aq.</t>
         </is>
       </c>
       <c r="H299" s="3" t="inlineStr">
@@ -26536,7 +26536,7 @@
       </c>
       <c r="G300" s="3" t="inlineStr">
         <is>
-          <t>Drospirenone/Estradiolethinyl</t>
+          <t>Drospirenone / Ethinylestradiol</t>
         </is>
       </c>
       <c r="H300" s="3" t="inlineStr">
@@ -26704,7 +26704,7 @@
       </c>
       <c r="G302" s="3" t="inlineStr">
         <is>
-          <t>Valproate (sodium) Sol'n</t>
+          <t>Valproate (sodium)</t>
         </is>
       </c>
       <c r="H302" s="3" t="inlineStr">
@@ -26789,7 +26789,7 @@
       </c>
       <c r="G303" s="3" t="inlineStr">
         <is>
-          <t>HemodialysisConc.(NaHCO3/NaCl)</t>
+          <t>Hemodialysis Conc.(Na HCO3 / Na Cl)</t>
         </is>
       </c>
       <c r="H303" s="3" t="inlineStr">
@@ -26856,7 +26856,7 @@
       </c>
       <c r="G304" s="3" t="inlineStr">
         <is>
-          <t>HemodialysisConc.(Sodium chloride/Potassium chloride/Magnesium chloride Hexahydrate/Calcium chloride dihydrate/Acetic acid/Dextrose)</t>
+          <t>Hemodialysis Conc.(Sodium Chloride / Potassium Chloride / Magnesiumchloride Hexahydrate / Calciumchloridedihydrate / Aceticacid / Dextrose)</t>
         </is>
       </c>
       <c r="H304" s="3" t="inlineStr">
@@ -26925,7 +26925,7 @@
       </c>
       <c r="G305" s="3" t="inlineStr">
         <is>
-          <t>HemodialysisConc.(NaCl/KCl/MgCl2.6H2O/CaCl2.2H2O/Acetic acid/Dextrose)</t>
+          <t>Hemodialysis Conc.(Na Cl / KCl / Mg Cl2.6H2O / Ca Cl2.2H2O / Aceticacid / Dextrose)</t>
         </is>
       </c>
       <c r="H305" s="3" t="inlineStr">
@@ -26994,7 +26994,7 @@
       </c>
       <c r="G306" s="3" t="inlineStr">
         <is>
-          <t>HemodialysisConc.(Sodium chloride/Potassium chloride/Magnesium chloride Hexahydrate/Calcium chloride dihydrate/Acetic acid/Dextrose)</t>
+          <t>Hemodialysis Conc.(Sodium Chloride / Potassium Chloride / Magnesiumchloride Hexahydrate / Calciumchloridedihydrate / Aceticacid / Dextrose)</t>
         </is>
       </c>
       <c r="H306" s="3" t="inlineStr">
@@ -27063,7 +27063,7 @@
       </c>
       <c r="G307" s="3" t="inlineStr">
         <is>
-          <t>Betamethasone (valerate)/Lidocaine (HCl)/Phenylephrine (HCl) Oint.</t>
+          <t>Betamethasone (valerate) / Lidocaine (HCl) / Phenylephrine (HCl) .</t>
         </is>
       </c>
       <c r="H307" s="3" t="inlineStr">
@@ -27387,7 +27387,7 @@
       </c>
       <c r="G311" s="3" t="inlineStr">
         <is>
-          <t>1,25-Dihydroxycalciferol</t>
+          <t>1 / 25-Dihydroxycalciferol</t>
         </is>
       </c>
       <c r="H311" s="3" t="inlineStr">
@@ -27480,7 +27480,7 @@
       </c>
       <c r="G312" s="3" t="inlineStr">
         <is>
-          <t>Brompheniramine (maleate)/Pseudoephedrine (HCl) Granules</t>
+          <t>Brompheniramine (maleate) / Pseudoephedrine (HCl)</t>
         </is>
       </c>
       <c r="H312" s="3" t="inlineStr">
@@ -27733,7 +27733,7 @@
       </c>
       <c r="G315" s="3" t="inlineStr">
         <is>
-          <t>IronhydroxidepolymaltosecomplexChewable</t>
+          <t>Iron Hydroxide Polymaltose Complex</t>
         </is>
       </c>
       <c r="H315" s="3" t="inlineStr">
@@ -27903,7 +27903,7 @@
       </c>
       <c r="G317" s="3" t="inlineStr">
         <is>
-          <t>HydrogenperoxideSol'n</t>
+          <t>Hydrogen Peroxide 3%</t>
         </is>
       </c>
       <c r="H317" s="3" t="inlineStr">
@@ -28146,7 +28146,7 @@
       </c>
       <c r="G320" s="3" t="inlineStr">
         <is>
-          <t>IpratropiumBrInhalationSol'n</t>
+          <t>Ipratropium Br Inhalation</t>
         </is>
       </c>
       <c r="H320" s="3" t="inlineStr">
@@ -28559,7 +28559,7 @@
       </c>
       <c r="G325" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride</t>
+          <t>Sodium Chloride</t>
         </is>
       </c>
       <c r="H325" s="3" t="inlineStr">
@@ -28628,7 +28628,7 @@
       </c>
       <c r="G326" s="3" t="inlineStr">
         <is>
-          <t>Sitagliptin phosphate</t>
+          <t>Sitagliptinphosphate</t>
         </is>
       </c>
       <c r="H326" s="3" t="inlineStr">
@@ -28895,7 +28895,7 @@
       </c>
       <c r="G329" s="3" t="inlineStr">
         <is>
-          <t>Empagliflozin/Metformin (HCl)</t>
+          <t>Empagliflozin / Metformin (HCl)</t>
         </is>
       </c>
       <c r="H329" s="3" t="inlineStr">
@@ -28989,7 +28989,7 @@
       </c>
       <c r="G330" s="3" t="inlineStr">
         <is>
-          <t>MiconazolenitrateVag.</t>
+          <t>Miconazole Nitrate</t>
         </is>
       </c>
       <c r="H330" s="3" t="inlineStr">
@@ -29075,7 +29075,7 @@
       </c>
       <c r="G331" s="3" t="inlineStr">
         <is>
-          <t>ChlorhexidinegluconateSol'n</t>
+          <t>Chlorhexidine Gluconate</t>
         </is>
       </c>
       <c r="H331" s="3" t="inlineStr">
@@ -29233,7 +29233,7 @@
       </c>
       <c r="G333" s="3" t="inlineStr">
         <is>
-          <t>Kaolin/Scopoliaextract/Albumin tannate/Bismuthsub carbonate</t>
+          <t>Kaolin / Scopolia Extract / Albumin Tannate / Bismuth Subcarbonate</t>
         </is>
       </c>
       <c r="H333" s="3" t="inlineStr">
@@ -29318,7 +29318,7 @@
       </c>
       <c r="G334" s="3" t="inlineStr">
         <is>
-          <t>Potassium chloride/Riboflavinphosphate sodium</t>
+          <t>Potassium Chloride / Riboflavinphosphatesodium</t>
         </is>
       </c>
       <c r="H334" s="3" t="inlineStr">
@@ -29403,7 +29403,7 @@
       </c>
       <c r="G335" s="3" t="inlineStr">
         <is>
-          <t>Calciumpolystyrenesulfonate Powder</t>
+          <t>Calciumpolystyrenesulfonate</t>
         </is>
       </c>
       <c r="H335" s="3" t="inlineStr">
@@ -29492,7 +29492,7 @@
       </c>
       <c r="G336" s="3" t="inlineStr">
         <is>
-          <t>PirenoxineOph.Susp.</t>
+          <t>Pirenoxine Oph..</t>
         </is>
       </c>
       <c r="H336" s="3" t="inlineStr">
@@ -29577,7 +29577,7 @@
       </c>
       <c r="G337" s="3" t="inlineStr">
         <is>
-          <t>DimethylPolysiloxane (Dimethicone)</t>
+          <t>Dimethyl Polysiloxane (Dimethicone)</t>
         </is>
       </c>
       <c r="H337" s="3" t="inlineStr">
@@ -30012,7 +30012,7 @@
       </c>
       <c r="G342" s="3" t="inlineStr">
         <is>
-          <t>L-Histidine/L-Lysine (acetate)/L-Threonine/L-Tryptophan/L-Tyrosine/Calcium-3-Methyl-2-Oxo-(valerate)/Calcium-4-Methyl-2-Oxo-(valerate)/Calcium-3-Methyl-2-Oxo-Butyrate/Calcium-2-Oxo-3-Phenyl-Propionate/Calcium-dl-2-Hydroxy-4-(Methyl-Thio)-Butyrate</t>
+          <t>L-Histidine / L-Lysine (acetate) / L-Threonine / L-Tryptophan / L-Tyrosine / Calcium-3-Methyl-2-Oxo-(valerate) / Calcium-4-Methyl-2-Oxo-(valerate) / Calcium-3-Methyl-2-Oxo-Butyrate / Calcium-2-Oxo-3-Phenyl-Propionate / Calcium-dl-2-Hydroxy-4-(Methyl-Thio)-Butyrate</t>
         </is>
       </c>
       <c r="H342" s="3" t="inlineStr">
@@ -30101,7 +30101,7 @@
       </c>
       <c r="G343" s="3" t="inlineStr">
         <is>
-          <t>Potassium gluconate</t>
+          <t>Potassiumgluconate</t>
         </is>
       </c>
       <c r="H343" s="3" t="inlineStr">
@@ -30279,7 +30279,7 @@
       </c>
       <c r="G345" s="3" t="inlineStr">
         <is>
-          <t>PsylliumHusk Powder</t>
+          <t>Psyllium Husk</t>
         </is>
       </c>
       <c r="H345" s="3" t="inlineStr">
@@ -30549,7 +30549,7 @@
       </c>
       <c r="G348" s="3" t="inlineStr">
         <is>
-          <t>LactobacillusBifidus Granules</t>
+          <t>Lactobacillus Bifidus</t>
         </is>
       </c>
       <c r="H348" s="3" t="inlineStr">
@@ -30638,7 +30638,7 @@
       </c>
       <c r="G349" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride/Sodium lactate/Calcium chloride/Potassium chloride</t>
+          <t>Sodium Chloride / Sodium Lactate / Calcium Chloride / Potassium Chloride</t>
         </is>
       </c>
       <c r="H349" s="3" t="inlineStr">
@@ -30894,7 +30894,7 @@
       </c>
       <c r="G352" s="3" t="inlineStr">
         <is>
-          <t>Lanthanum (carbonate dihydrate)</t>
+          <t>Lanthanum (carbonatedihydrate)</t>
         </is>
       </c>
       <c r="H352" s="3" t="inlineStr">
@@ -31562,7 +31562,7 @@
       </c>
       <c r="G360" s="3" t="inlineStr">
         <is>
-          <t>LevetiracetamOralSol'n</t>
+          <t>Levetiracetam Oral</t>
         </is>
       </c>
       <c r="H360" s="3" t="inlineStr">
@@ -31651,7 +31651,7 @@
       </c>
       <c r="G361" s="3" t="inlineStr">
         <is>
-          <t>Levofloxacin hemihydrate</t>
+          <t>Levofloxacinhemihydrate</t>
         </is>
       </c>
       <c r="H361" s="3" t="inlineStr">
@@ -31740,7 +31740,7 @@
       </c>
       <c r="G362" s="3" t="inlineStr">
         <is>
-          <t>Levofloxacin hemihydrate</t>
+          <t>Levofloxacinhemihydrate</t>
         </is>
       </c>
       <c r="H362" s="3" t="inlineStr">
@@ -31983,7 +31983,7 @@
       </c>
       <c r="G365" s="3" t="inlineStr">
         <is>
-          <t>Epinephrine/Lidocaine (HCl)</t>
+          <t>Epinephrine / Lidocaine (HCl)</t>
         </is>
       </c>
       <c r="H365" s="3" t="inlineStr">
@@ -32072,7 +32072,7 @@
       </c>
       <c r="G366" s="3" t="inlineStr">
         <is>
-          <t>Lithium carbonate</t>
+          <t>Lithiumcarbonate</t>
         </is>
       </c>
       <c r="H366" s="3" t="inlineStr">
@@ -32157,7 +32157,7 @@
       </c>
       <c r="G367" s="3" t="inlineStr">
         <is>
-          <t>HyoscineButyl bromide (ButylscopolamineBr)</t>
+          <t>Hyoscine Butylbromide (Butylscopolamine Br)</t>
         </is>
       </c>
       <c r="H367" s="3" t="inlineStr">
@@ -32246,7 +32246,7 @@
       </c>
       <c r="G368" s="3" t="inlineStr">
         <is>
-          <t>Glycyrrhizafluidextract/Antimonypotassium tartrate/OpiumtinctureLiq.</t>
+          <t>Glycyrrhizafluidextract / Antimonypotassiumtartrate / Opiumtincture Liq.</t>
         </is>
       </c>
       <c r="H368" s="3" t="inlineStr">
@@ -32509,7 +32509,7 @@
       </c>
       <c r="G371" s="3" t="inlineStr">
         <is>
-          <t>Edoxabantosilate</t>
+          <t>Edoxaban Tosilate</t>
         </is>
       </c>
       <c r="H371" s="3" t="inlineStr">
@@ -32598,7 +32598,7 @@
       </c>
       <c r="G372" s="3" t="inlineStr">
         <is>
-          <t>Edoxabantosilate</t>
+          <t>Edoxaban Tosilate</t>
         </is>
       </c>
       <c r="H372" s="3" t="inlineStr">
@@ -32951,7 +32951,7 @@
       </c>
       <c r="G376" s="3" t="inlineStr">
         <is>
-          <t>Loratadine/Pseudoephedrine (sulfate)</t>
+          <t>Loratadine / Pseudoephedrine (sulfate)</t>
         </is>
       </c>
       <c r="H376" s="3" t="inlineStr">
@@ -33214,7 +33214,7 @@
       </c>
       <c r="G379" s="3" t="inlineStr">
         <is>
-          <t>Silymarin/Niacinamide/Thiamine (Vit.B1) hydrochloride/Riboflavin (Vit.B2)/Pyridoxine (Vit.B6)(HCl)/Cyanocobalamin (Vit.B12)/Pantothenate calcium</t>
+          <t>Silymarin / Niacinamide / Thiamine (Vit. B1) hydrochloride / Riboflavin (Vit. B2) / Pyridoxine (Vit. B6)(HCl) / Cyanocobalamin (Vit. B12) / Pantothenatecalcium</t>
         </is>
       </c>
       <c r="H379" s="3" t="inlineStr">
@@ -33372,7 +33372,7 @@
       </c>
       <c r="G381" s="3" t="inlineStr">
         <is>
-          <t>Acetylsalicylic acid (Aspirin)</t>
+          <t>Acetylsalicylic Acid (Aspirin)</t>
         </is>
       </c>
       <c r="H381" s="3" t="inlineStr">
@@ -33457,7 +33457,7 @@
       </c>
       <c r="G382" s="3" t="inlineStr">
         <is>
-          <t>Rifampin/Isoniazid</t>
+          <t>Rifampin / Isoniazid</t>
         </is>
       </c>
       <c r="H382" s="3" t="inlineStr">
@@ -33542,7 +33542,7 @@
       </c>
       <c r="G383" s="3" t="inlineStr">
         <is>
-          <t>Levodopa/Benserazide (HCl)</t>
+          <t>Levodopa / Benserazide (HCl)</t>
         </is>
       </c>
       <c r="H383" s="3" t="inlineStr">
@@ -33631,7 +33631,7 @@
       </c>
       <c r="G384" s="3" t="inlineStr">
         <is>
-          <t>Magnesium oxide</t>
+          <t>Magnesium Oxide</t>
         </is>
       </c>
       <c r="H384" s="3" t="inlineStr">
@@ -33724,7 +33724,7 @@
       </c>
       <c r="G385" s="3" t="inlineStr">
         <is>
-          <t>Magnesium sulfate</t>
+          <t>Magnesium Sulfate</t>
         </is>
       </c>
       <c r="H385" s="3" t="inlineStr">
@@ -33813,7 +33813,7 @@
       </c>
       <c r="G386" s="3" t="inlineStr">
         <is>
-          <t>BupivacaineHCl (monohydrate)</t>
+          <t>Bupivacaine HCl (monohydrate)</t>
         </is>
       </c>
       <c r="H386" s="3" t="inlineStr">
@@ -33886,7 +33886,7 @@
       </c>
       <c r="G387" s="3" t="inlineStr">
         <is>
-          <t>BupivacaineHCl (monohydrate)</t>
+          <t>Bupivacaine HCl (monohydrate)</t>
         </is>
       </c>
       <c r="H387" s="3" t="inlineStr">
@@ -33979,7 +33979,7 @@
       </c>
       <c r="G388" s="3" t="inlineStr">
         <is>
-          <t>BupivacaineHCl (monohydrate) SpinalHeavy</t>
+          <t>Bupivacaine HCl (monohydrate) Spinal Heavy</t>
         </is>
       </c>
       <c r="H388" s="3" t="inlineStr">
@@ -34052,7 +34052,7 @@
       </c>
       <c r="G389" s="3" t="inlineStr">
         <is>
-          <t>Glecaprevir/Pibrentasvir</t>
+          <t>Glecaprevir / Pibrentasvir</t>
         </is>
       </c>
       <c r="H389" s="3" t="inlineStr">
@@ -34380,7 +34380,7 @@
       </c>
       <c r="G393" s="3" t="inlineStr">
         <is>
-          <t>Dextromethorphan (HBr)/Lysozyme chloride/Potassium cresolsulfonate</t>
+          <t>Dextromethorphan (HBr) / Lysozymechloride / Potassiumcresolsulfonate</t>
         </is>
       </c>
       <c r="H393" s="3" t="inlineStr">
@@ -34550,7 +34550,7 @@
       </c>
       <c r="G395" s="3" t="inlineStr">
         <is>
-          <t>Megestrol (acetate) OralSusp.</t>
+          <t>Megestrol (acetate) Oral .</t>
         </is>
       </c>
       <c r="H395" s="3" t="inlineStr">
@@ -34813,7 +34813,7 @@
       </c>
       <c r="G398" s="3" t="inlineStr">
         <is>
-          <t>Meropenem trihydrate</t>
+          <t>Meropenemtrihydrate</t>
         </is>
       </c>
       <c r="H398" s="3" t="inlineStr">
@@ -34902,7 +34902,7 @@
       </c>
       <c r="G399" s="3" t="inlineStr">
         <is>
-          <t>Methylprednisolone sodium succinate</t>
+          <t>Methylprednisolonesodiumsuccinate</t>
         </is>
       </c>
       <c r="H399" s="3" t="inlineStr">
@@ -35505,7 +35505,7 @@
       </c>
       <c r="G406" s="3" t="inlineStr">
         <is>
-          <t>Dioctyl sodium sulfo succinate/Bisacodyl/Sennoside</t>
+          <t>Dioctyl sodium sulfosuccinate / Bisacodyl / Sennoside</t>
         </is>
       </c>
       <c r="H406" s="3" t="inlineStr">
@@ -35570,7 +35570,7 @@
       </c>
       <c r="G407" s="3" t="inlineStr">
         <is>
-          <t>Desmopressin (acetate trihydrate)</t>
+          <t>Desmopressin (acetatetrihydrate)</t>
         </is>
       </c>
       <c r="H407" s="3" t="inlineStr">
@@ -35659,7 +35659,7 @@
       </c>
       <c r="G408" s="3" t="inlineStr">
         <is>
-          <t>Pramipexole dihydrochloride</t>
+          <t>Pramipexoledihydrochloride</t>
         </is>
       </c>
       <c r="H408" s="3" t="inlineStr">
@@ -35837,7 +35837,7 @@
       </c>
       <c r="G410" s="3" t="inlineStr">
         <is>
-          <t>LevonorgestrelIntrauterineSystem</t>
+          <t>Levonorgestrel Intrauterine System</t>
         </is>
       </c>
       <c r="H410" s="3" t="inlineStr">
@@ -35926,7 +35926,7 @@
       </c>
       <c r="G411" s="3" t="inlineStr">
         <is>
-          <t>ClostridiumButyricumMiyairi</t>
+          <t>Clostridium Butyricum Miyairi</t>
         </is>
       </c>
       <c r="H411" s="3" t="inlineStr">
@@ -36098,7 +36098,7 @@
       </c>
       <c r="G413" s="3" t="inlineStr">
         <is>
-          <t>Flupentixol (2HCl)/Melitracen (HCl)</t>
+          <t>Flupentixol (2HCl) / Melitracen (HCl)</t>
         </is>
       </c>
       <c r="H413" s="3" t="inlineStr">
@@ -36268,7 +36268,7 @@
       </c>
       <c r="G415" s="3" t="inlineStr">
         <is>
-          <t>MometasoneNasal Spray</t>
+          <t>Mometasone</t>
         </is>
       </c>
       <c r="H415" s="3" t="inlineStr">
@@ -36349,7 +36349,7 @@
       </c>
       <c r="G416" s="3" t="inlineStr">
         <is>
-          <t>L-Alanine/L-Arginine/L-Aspartic acid/L-Cysteine/L-Glutamic acid/L-Histidine/L-Isoleucine/L-Leucine/Lysine acetate/L-Methionine/L-Phenylalanine/L-Proline/L-Serine/L-Threonine/L-Tryptophan/L-Tyrosine/L-Valine</t>
+          <t>L-Alanine / L-Arginine / L-Asparticacid / L-Cysteine / L-Glutamicacid / L-Histidine / L-Isoleucine / L-Leucine / Lysineacetate / L-Methionine / L-Phenylalanine / L-Proline / L-Serine / L-Threonine / L-Tryptophan / L-Tyrosine / L-Valine</t>
         </is>
       </c>
       <c r="H416" s="3" t="inlineStr">
@@ -36434,7 +36434,7 @@
       </c>
       <c r="G417" s="3" t="inlineStr">
         <is>
-          <t>Mosapride (citrate dihydrate)</t>
+          <t>Mosapride (citratedihydrate)</t>
         </is>
       </c>
       <c r="H417" s="3" t="inlineStr">
@@ -36503,7 +36503,7 @@
       </c>
       <c r="G418" s="3" t="inlineStr">
         <is>
-          <t>Moxifloxacin (HCl) infusionSol'n</t>
+          <t>Moxifloxacin (HCl) infusion</t>
         </is>
       </c>
       <c r="H418" s="3" t="inlineStr">
@@ -36677,7 +36677,7 @@
       </c>
       <c r="G420" s="3" t="inlineStr">
         <is>
-          <t>Neomycin (Fradiomycin)/Nystatin (sulfate)/Triamcinoloneacetonide/Gramicidin Cream</t>
+          <t>Neomycin (Fradiomycin) / Nystatin (sulfate) / Triamcinoloneacetonide / Gramicidin</t>
         </is>
       </c>
       <c r="H420" s="3" t="inlineStr">
@@ -36762,7 +36762,7 @@
       </c>
       <c r="G421" s="3" t="inlineStr">
         <is>
-          <t>Neomycin (Fradiomycin)/Nystatin/Triamcinoloneacetonide/GramicidinOtic.Drops</t>
+          <t>Neomycin (Fradiomycin) / Nystatin / Triamcinoloneacetonide / Gramicidin Otic.Drops</t>
         </is>
       </c>
       <c r="H421" s="3" t="inlineStr">
@@ -37094,7 +37094,7 @@
       </c>
       <c r="G425" s="3" t="inlineStr">
         <is>
-          <t>L-Isoleucine/L-Leucine/L-Lysinemonoacetate/L-Methioinine/Acetylcysteine/L-Phenylalanine/L-Threonine/L-Tryptophan/L-Valine/Arginine/L-Histidine/Aminoacetic acid/L-Alanine/L-Proline/L-Serine/L-Malic acid</t>
+          <t>L-Isoleucine / L-Leucine / L-Lysinemonoacetate / L-Methioinine / Acetylcysteine / L-Phenylalanine / L-Threonine / L-Tryptophan / L-Valine / Arginine / L-Histidine / Aminoacetic Acid / L-Alanine / L-Proline / L-Serine / L-Malicacid</t>
         </is>
       </c>
       <c r="H425" s="3" t="inlineStr">
@@ -37179,7 +37179,7 @@
       </c>
       <c r="G426" s="3" t="inlineStr">
         <is>
-          <t>Darbepoetinalfa</t>
+          <t>Darbepoetin Alfa</t>
         </is>
       </c>
       <c r="H426" s="3" t="inlineStr">
@@ -37276,7 +37276,7 @@
       </c>
       <c r="G427" s="3" t="inlineStr">
         <is>
-          <t>RotigotineTransdermalPatch</t>
+          <t>Rotigotine Transdermal Patch</t>
         </is>
       </c>
       <c r="H427" s="3" t="inlineStr">
@@ -37543,7 +37543,7 @@
       </c>
       <c r="G430" s="3" t="inlineStr">
         <is>
-          <t>NicotineChewingGum</t>
+          <t>Nicotine Chewing Gum</t>
         </is>
       </c>
       <c r="H430" s="3" t="inlineStr">
@@ -37626,7 +37626,7 @@
       </c>
       <c r="G431" s="3" t="inlineStr">
         <is>
-          <t>NicotineTTS30</t>
+          <t>Nicotine TTS30</t>
         </is>
       </c>
       <c r="H431" s="3" t="inlineStr">
@@ -37952,7 +37952,7 @@
       </c>
       <c r="G435" s="3" t="inlineStr">
         <is>
-          <t>NimodipineInfusionSol'n</t>
+          <t>Nimodipine Infusion</t>
         </is>
       </c>
       <c r="H435" s="3" t="inlineStr">
@@ -38041,7 +38041,7 @@
       </c>
       <c r="G436" s="3" t="inlineStr">
         <is>
-          <t>TriamcinoloneacetonideInOralBase Gel</t>
+          <t>Triamcinolone Acetonide (Oral Base)</t>
         </is>
       </c>
       <c r="H436" s="3" t="inlineStr">
@@ -38300,7 +38300,7 @@
       </c>
       <c r="G439" s="3" t="inlineStr">
         <is>
-          <t>Tamoxifen citrate</t>
+          <t>Tamoxifencitrate</t>
         </is>
       </c>
       <c r="H439" s="3" t="inlineStr">
@@ -38555,7 +38555,7 @@
       </c>
       <c r="G442" s="3" t="inlineStr">
         <is>
-          <t>SodiumchlorideforWash</t>
+          <t>Sodium Chloride (Irrigation / Wash 0.9%)</t>
         </is>
       </c>
       <c r="H442" s="3" t="inlineStr">
@@ -38785,7 +38785,7 @@
       </c>
       <c r="G445" s="3" t="inlineStr">
         <is>
-          <t>InsulinAspart/InsulinAspartProtamine</t>
+          <t>Insulin Aspart / Insulin Aspart Protamine</t>
         </is>
       </c>
       <c r="H445" s="3" t="inlineStr">
@@ -38878,7 +38878,7 @@
       </c>
       <c r="G446" s="3" t="inlineStr">
         <is>
-          <t>InsulinAspart</t>
+          <t>Insulin Aspart</t>
         </is>
       </c>
       <c r="H446" s="3" t="inlineStr">
@@ -39138,7 +39138,7 @@
       </c>
       <c r="G449" s="3" t="inlineStr">
         <is>
-          <t>NeostigminemethylsulfateOphSol'n</t>
+          <t>Neostigmine Methylsulfate</t>
         </is>
       </c>
       <c r="H449" s="3" t="inlineStr">
@@ -39228,7 +39228,7 @@
       </c>
       <c r="G450" s="3" t="inlineStr">
         <is>
-          <t>Emtricitabine/Rilpivirine/Tenofoviralafenamide</t>
+          <t>Emtricitabine / Rilpivirine / Tenofovir Alafenamide</t>
         </is>
       </c>
       <c r="H450" s="3" t="inlineStr">
@@ -39317,7 +39317,7 @@
       </c>
       <c r="G451" s="3" t="inlineStr">
         <is>
-          <t>Nintedanibethanesulfonate</t>
+          <t>Nintedanib Ethanesulfonate</t>
         </is>
       </c>
       <c r="H451" s="3" t="inlineStr">
@@ -39402,7 +39402,7 @@
       </c>
       <c r="G452" s="3" t="inlineStr">
         <is>
-          <t>OfloxacinOtic.Sol'n</t>
+          <t>Ofloxacin Otic.</t>
         </is>
       </c>
       <c r="H452" s="3" t="inlineStr">
@@ -39491,7 +39491,7 @@
       </c>
       <c r="G453" s="3" t="inlineStr">
         <is>
-          <t>RisperidoneSusp.</t>
+          <t>Risperidone .</t>
         </is>
       </c>
       <c r="H453" s="3" t="inlineStr">
@@ -39576,7 +39576,7 @@
       </c>
       <c r="G454" s="3" t="inlineStr">
         <is>
-          <t>OlanzapineOralDispersible</t>
+          <t>Olanzapine</t>
         </is>
       </c>
       <c r="H454" s="3" t="inlineStr">
@@ -40724,7 +40724,7 @@
       </c>
       <c r="G467" s="3" t="inlineStr">
         <is>
-          <t>Pancreatin/Metoclopramide (HCl)</t>
+          <t>Pancreatin / Metoclopramide (HCl)</t>
         </is>
       </c>
       <c r="H467" s="3" t="inlineStr">
@@ -40813,7 +40813,7 @@
       </c>
       <c r="G468" s="3" t="inlineStr">
         <is>
-          <t>Potassium chloride/Sodium chloride/Borax/Sodium biphosphate/Benzalkonium chloride/BoricacidEye Lotion</t>
+          <t>Potassium Chloride / Sodium Chloride / Borax / Sodiumbiphosphate / Benzalkoniumchloride / Boricacid Eye</t>
         </is>
       </c>
       <c r="H468" s="3" t="inlineStr">
@@ -40902,7 +40902,7 @@
       </c>
       <c r="G469" s="3" t="inlineStr">
         <is>
-          <t>Mesalazine Granules</t>
+          <t>Mesalazine</t>
         </is>
       </c>
       <c r="H469" s="3" t="inlineStr">
@@ -41149,7 +41149,7 @@
       </c>
       <c r="G472" s="3" t="inlineStr">
         <is>
-          <t>RisperidoneOralSol'n</t>
+          <t>Risperidone Oral</t>
         </is>
       </c>
       <c r="H472" s="3" t="inlineStr">
@@ -41501,7 +41501,7 @@
       </c>
       <c r="G476" s="3" t="inlineStr">
         <is>
-          <t>Phytonadione (=Phytomenadione)(Vit.K1)</t>
+          <t>Phytonadione (=Phytomenadione)(Vit. K1)</t>
         </is>
       </c>
       <c r="H476" s="3" t="inlineStr">
@@ -41667,7 +41667,7 @@
       </c>
       <c r="G478" s="3" t="inlineStr">
         <is>
-          <t>Piperacillin (sodium)/Tazobactam (sodium)</t>
+          <t>Piperacillin (sodium) / Tazobactam (sodium)</t>
         </is>
       </c>
       <c r="H478" s="3" t="inlineStr">
@@ -42015,7 +42015,7 @@
       </c>
       <c r="G482" s="3" t="inlineStr">
         <is>
-          <t>Desmopressin (acetate trihydrate)</t>
+          <t>Desmopressin (acetatetrihydrate)</t>
         </is>
       </c>
       <c r="H482" s="3" t="inlineStr">
@@ -42100,7 +42100,7 @@
       </c>
       <c r="G483" s="3" t="inlineStr">
         <is>
-          <t>PolicresulenVag.Supp.</t>
+          <t>Policresulen Vag..</t>
         </is>
       </c>
       <c r="H483" s="3" t="inlineStr">
@@ -42273,7 +42273,7 @@
       </c>
       <c r="G485" s="3" t="inlineStr">
         <is>
-          <t>Mefenamic acid</t>
+          <t>Mefenamic Acid</t>
         </is>
       </c>
       <c r="H485" s="3" t="inlineStr">
@@ -42625,7 +42625,7 @@
       </c>
       <c r="G489" s="3" t="inlineStr">
         <is>
-          <t>Fenofibrate/Pravastatin (sodium)</t>
+          <t>Fenofibrate / Pravastatin (sodium)</t>
         </is>
       </c>
       <c r="H489" s="3" t="inlineStr">
@@ -42965,7 +42965,7 @@
       </c>
       <c r="G493" s="3" t="inlineStr">
         <is>
-          <t>ConjugatedEstrogenVag.Cream</t>
+          <t>Conjugated Estrogen Vag.</t>
         </is>
       </c>
       <c r="H493" s="3" t="inlineStr">
@@ -43759,7 +43759,7 @@
       </c>
       <c r="G502" s="3" t="inlineStr">
         <is>
-          <t>Dapagliflozin/Saxagliptin</t>
+          <t>Dapagliflozin / Saxagliptin</t>
         </is>
       </c>
       <c r="H502" s="3" t="inlineStr">
@@ -44308,7 +44308,7 @@
       </c>
       <c r="G508" s="3" t="inlineStr">
         <is>
-          <t>Succinylcholine chloride</t>
+          <t>Succinylcholinechloride</t>
         </is>
       </c>
       <c r="H508" s="3" t="inlineStr">
@@ -44398,7 +44398,7 @@
       </c>
       <c r="G509" s="3" t="inlineStr">
         <is>
-          <t>Fluticasonefuroate/VilanterolInhalation Powder</t>
+          <t>Fluticasone Furoate / Vilanterol Trifenatate</t>
         </is>
       </c>
       <c r="H509" s="3" t="inlineStr">
@@ -45002,7 +45002,7 @@
       </c>
       <c r="G516" s="3" t="inlineStr">
         <is>
-          <t>Rizatriptan benzoate</t>
+          <t>Rizatriptanbenzoate</t>
         </is>
       </c>
       <c r="H516" s="3" t="inlineStr">
@@ -45180,7 +45180,7 @@
       </c>
       <c r="G518" s="3" t="inlineStr">
         <is>
-          <t>Sodium bicarbonate</t>
+          <t>Sodium Bicarbonate</t>
         </is>
       </c>
       <c r="H518" s="3" t="inlineStr">
@@ -45265,7 +45265,7 @@
       </c>
       <c r="G519" s="3" t="inlineStr">
         <is>
-          <t>AesculushippocastanumLextract</t>
+          <t>Aesculus Hippocastanum Extract</t>
         </is>
       </c>
       <c r="H519" s="3" t="inlineStr">
@@ -45435,7 +45435,7 @@
       </c>
       <c r="G521" s="3" t="inlineStr">
         <is>
-          <t>Clindamycin (phosphate) Gel</t>
+          <t>Clindamycin (phosphate)</t>
         </is>
       </c>
       <c r="H521" s="3" t="inlineStr">
@@ -45699,7 +45699,7 @@
       </c>
       <c r="G524" s="3" t="inlineStr">
         <is>
-          <t>InsulinAspart/InsulinDegludec</t>
+          <t>Insulin Aspart / Insulin Degludec</t>
         </is>
       </c>
       <c r="H524" s="3" t="inlineStr">
@@ -45963,7 +45963,7 @@
       </c>
       <c r="G527" s="3" t="inlineStr">
         <is>
-          <t>SalicylicacidOint.</t>
+          <t>Salicylicacid .</t>
         </is>
       </c>
       <c r="H527" s="3" t="inlineStr">
@@ -46140,7 +46140,7 @@
       </c>
       <c r="G529" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride</t>
+          <t>Sodium Chloride</t>
         </is>
       </c>
       <c r="H529" s="3" t="inlineStr">
@@ -46298,7 +46298,7 @@
       </c>
       <c r="G531" s="3" t="inlineStr">
         <is>
-          <t>CyanocobalamineOph.Sol'n</t>
+          <t>Cyanocobalamine Oph.</t>
         </is>
       </c>
       <c r="H531" s="3" t="inlineStr">
@@ -46383,7 +46383,7 @@
       </c>
       <c r="G532" s="3" t="inlineStr">
         <is>
-          <t>IbuprofenOralSusp.</t>
+          <t>Ibuprofen Oral .</t>
         </is>
       </c>
       <c r="H532" s="3" t="inlineStr">
@@ -46468,7 +46468,7 @@
       </c>
       <c r="G533" s="3" t="inlineStr">
         <is>
-          <t>SucralfateOralSusp.</t>
+          <t>Sucralfate Oral .</t>
         </is>
       </c>
       <c r="H533" s="3" t="inlineStr">
@@ -46557,7 +46557,7 @@
       </c>
       <c r="G534" s="3" t="inlineStr">
         <is>
-          <t>SennosideA+B</t>
+          <t>Sennoside A + B</t>
         </is>
       </c>
       <c r="H534" s="3" t="inlineStr">
@@ -46626,7 +46626,7 @@
       </c>
       <c r="G535" s="3" t="inlineStr">
         <is>
-          <t>Betamethasone (dipropionate) Sol'n</t>
+          <t>Betamethasone (dipropionate)</t>
         </is>
       </c>
       <c r="H535" s="3" t="inlineStr">
@@ -46715,7 +46715,7 @@
       </c>
       <c r="G536" s="3" t="inlineStr">
         <is>
-          <t>Fluticasone/Salmeterol Evohaler</t>
+          <t>Fluticasone / Salmeterol Evohaler</t>
         </is>
       </c>
       <c r="H536" s="3" t="inlineStr">
@@ -46873,7 +46873,7 @@
       </c>
       <c r="G538" s="3" t="inlineStr">
         <is>
-          <t>Amlodipine (besylate)/Olmesartanmedoxomil</t>
+          <t>Amlodipine (besylate) / Olmesartanmedoxomil</t>
         </is>
       </c>
       <c r="H538" s="3" t="inlineStr">
@@ -46963,7 +46963,7 @@
       </c>
       <c r="G539" s="3" t="inlineStr">
         <is>
-          <t>Amlodipine (besylate)/Olmesartanmedoxomil/Hydrochlorothiazide</t>
+          <t>Amlodipine (besylate) / Olmesartanmedoxomil / Hydrochlorothiazide</t>
         </is>
       </c>
       <c r="H539" s="3" t="inlineStr">
@@ -47052,7 +47052,7 @@
       </c>
       <c r="G540" s="3" t="inlineStr">
         <is>
-          <t>VaricellaZosterVirusglycoproteinE</t>
+          <t>Varicella Zoster Virus Glycoprotein E</t>
         </is>
       </c>
       <c r="H540" s="3" t="inlineStr">
@@ -47228,7 +47228,7 @@
       </c>
       <c r="G542" s="3" t="inlineStr">
         <is>
-          <t>Sulfadiazinesilver Cream</t>
+          <t>Silver Sulfadiazine</t>
         </is>
       </c>
       <c r="H542" s="3" t="inlineStr">
@@ -47313,7 +47313,7 @@
       </c>
       <c r="G543" s="3" t="inlineStr">
         <is>
-          <t>Povidone-IodineAlc.Sol'n</t>
+          <t>Povidone-Iodine Alc.</t>
         </is>
       </c>
       <c r="H543" s="3" t="inlineStr">
@@ -47382,7 +47382,7 @@
       </c>
       <c r="G544" s="3" t="inlineStr">
         <is>
-          <t>Povidone-IodineOint.</t>
+          <t>Povidone-Iodine .</t>
         </is>
       </c>
       <c r="H544" s="3" t="inlineStr">
@@ -47746,7 +47746,7 @@
       </c>
       <c r="G548" s="3" t="inlineStr">
         <is>
-          <t>Mesna (Sodium2-Mercaptoethanesulphonate) Inh.Sol'n</t>
+          <t>Mesna (Sodium2-Mercaptoethanesulphonate) Inh.</t>
         </is>
       </c>
       <c r="H548" s="3" t="inlineStr">
@@ -47827,7 +47827,7 @@
       </c>
       <c r="G549" s="3" t="inlineStr">
         <is>
-          <t>Dioctahedralsmectite (diosmectite) PowderOralSusp.</t>
+          <t>Dioctahedralsmectite (diosmectite) Oral .</t>
         </is>
       </c>
       <c r="H549" s="3" t="inlineStr">
@@ -47914,7 +47914,7 @@
       </c>
       <c r="G550" s="3" t="inlineStr">
         <is>
-          <t>Sodium acetate trihydrate/Calcium chloride dihydrate/Potassium chloride/Glucose/Soybean oil/Fish-Oilrichinomega-3acids/Alanine/Arginine/Histidine/Isoleucine/Leucine/Lysine/Methionine/Phenylalanine/Proline/Serine/Threonine/Tryptophan/Tyrosine/Valine/Glycine (=Aminoacetic acid)(=glycocoll)/Magnesiumsulfateheptahydrate/Triglyceridesmediumchain/Taurine (=Aminoethylsulfonic acid)/Sodiumglycero phosphate/Zinc sulfate7H2O/Olive oil</t>
+          <t>Soybean Oil / Medium-Chain Triglycerides / Olive Oil / Fish Oil</t>
         </is>
       </c>
       <c r="H550" s="3" t="inlineStr">
@@ -47999,7 +47999,7 @@
       </c>
       <c r="G551" s="3" t="inlineStr">
         <is>
-          <t>Soybean oil/Fish-oil/Triglycerides/Olive oil</t>
+          <t>Soybean Oil / Fish-oil / Triglycerides / Olive Oil</t>
         </is>
       </c>
       <c r="H551" s="3" t="inlineStr">
@@ -48084,7 +48084,7 @@
       </c>
       <c r="G552" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride</t>
+          <t>Sodium Chloride</t>
         </is>
       </c>
       <c r="H552" s="3" t="inlineStr">
@@ -48157,7 +48157,7 @@
       </c>
       <c r="G553" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride</t>
+          <t>Sodium Chloride</t>
         </is>
       </c>
       <c r="H553" s="3" t="inlineStr">
@@ -48230,7 +48230,7 @@
       </c>
       <c r="G554" s="3" t="inlineStr">
         <is>
-          <t>Sodium bicarbonate</t>
+          <t>Sodium Bicarbonate</t>
         </is>
       </c>
       <c r="H554" s="3" t="inlineStr">
@@ -48319,7 +48319,7 @@
       </c>
       <c r="G555" s="3" t="inlineStr">
         <is>
-          <t>Ethanol/1-Propanol</t>
+          <t>Ethanol / 1-Propanol</t>
         </is>
       </c>
       <c r="H555" s="3" t="inlineStr">
@@ -48386,7 +48386,7 @@
       </c>
       <c r="G556" s="3" t="inlineStr">
         <is>
-          <t>Methylprednisolone sodium succinate</t>
+          <t>Methylprednisolonesodiumsuccinate</t>
         </is>
       </c>
       <c r="H556" s="3" t="inlineStr">
@@ -48556,7 +48556,7 @@
       </c>
       <c r="G558" s="3" t="inlineStr">
         <is>
-          <t>TiotropiumBr/Olodaterol (HCl) Sol'nfor Inhalation</t>
+          <t>Tiotropium Br / Olodaterol (HCl) Sol'nfor Inhalation</t>
         </is>
       </c>
       <c r="H558" s="3" t="inlineStr">
@@ -48641,7 +48641,7 @@
       </c>
       <c r="G559" s="3" t="inlineStr">
         <is>
-          <t>TiotropiumBrSol'nfor Inhalation</t>
+          <t>Tiotropium Br Sol'nfor Inhalation</t>
         </is>
       </c>
       <c r="H559" s="3" t="inlineStr">
@@ -48900,7 +48900,7 @@
       </c>
       <c r="G562" s="3" t="inlineStr">
         <is>
-          <t>Carbidopa/Levodopa/Entacapone</t>
+          <t>Carbidopa / Levodopa / Entacapone</t>
         </is>
       </c>
       <c r="H562" s="3" t="inlineStr">
@@ -49078,7 +49078,7 @@
       </c>
       <c r="G564" s="3" t="inlineStr">
         <is>
-          <t>CellulaseAP3/Biodiastase2000/LipaseAP6/Prozyme6</t>
+          <t>Cellulase AP3 / Biodiastase2000 / Lipase AP6 / Prozyme6</t>
         </is>
       </c>
       <c r="H564" s="3" t="inlineStr">
@@ -49163,7 +49163,7 @@
       </c>
       <c r="G565" s="3" t="inlineStr">
         <is>
-          <t>Oxethazaine/Polymi gel (Alhydr oxide+CaCO3+MgCO3)</t>
+          <t>Oxethazaine / Polymigel (Alhydroxide + Ca CO3 + Mg CO3)</t>
         </is>
       </c>
       <c r="H565" s="3" t="inlineStr">
@@ -49339,7 +49339,7 @@
       </c>
       <c r="G567" s="3" t="inlineStr">
         <is>
-          <t>Glycyrrhizinmonoammonium/Glycine (Aminoacetic acid)(Glycocoll)/L-Cycteine (HCl)</t>
+          <t>Glycyrrhizinmonoammonium / Glycine (Aminoacetic Acid)(Glycocoll) / L-Cycteine (HCl)</t>
         </is>
       </c>
       <c r="H567" s="3" t="inlineStr">
@@ -49509,7 +49509,7 @@
       </c>
       <c r="G569" s="3" t="inlineStr">
         <is>
-          <t>Repaglinide</t>
+          <t>Insulin Aspart Protamine / Insulin Aspart</t>
         </is>
       </c>
       <c r="H569" s="3" t="inlineStr">
@@ -49754,7 +49754,7 @@
       </c>
       <c r="G572" s="3" t="inlineStr">
         <is>
-          <t>Budesonide/Formoterol (fumarate2H2O) Rapihaler</t>
+          <t>Budesonide / Formoterol (fumarate2H2O) Rapihaler</t>
         </is>
       </c>
       <c r="H572" s="3" t="inlineStr">
@@ -49839,7 +49839,7 @@
       </c>
       <c r="G573" s="3" t="inlineStr">
         <is>
-          <t>Paliperidone palmitate Susp.</t>
+          <t>Paliperidone palmitate .</t>
         </is>
       </c>
       <c r="H573" s="3" t="inlineStr">
@@ -49908,7 +49908,7 @@
       </c>
       <c r="G574" s="3" t="inlineStr">
         <is>
-          <t>Estradiol (valerate)(Tab.1)/Estradiol (valerate)(Tab.2)/Medroxyprogesterone (acetate)(Tab.3)</t>
+          <t>Estradiol (valerate)(Tab.1) / Estradiol (valerate)(Tab.2) / Medroxyprogesterone (acetate)(Tab.3)</t>
         </is>
       </c>
       <c r="H574" s="3" t="inlineStr">
@@ -50153,7 +50153,7 @@
       </c>
       <c r="G577" s="3" t="inlineStr">
         <is>
-          <t>PiracetamGranulesforOralSol'n</t>
+          <t>Piracetam Granulesfor Oral</t>
         </is>
       </c>
       <c r="H577" s="3" t="inlineStr">
@@ -50501,7 +50501,7 @@
       </c>
       <c r="G581" s="3" t="inlineStr">
         <is>
-          <t>Tafluprost Oph. Sol'n</t>
+          <t>Tafluprost Oph.</t>
         </is>
       </c>
       <c r="H581" s="3" t="inlineStr">
@@ -50677,7 +50677,7 @@
       </c>
       <c r="G583" s="3" t="inlineStr">
         <is>
-          <t>NemonoxacinMalate Hemihydrate</t>
+          <t>Nemonoxacin Malate Hemihydrate</t>
         </is>
       </c>
       <c r="H583" s="3" t="inlineStr">
@@ -50770,7 +50770,7 @@
       </c>
       <c r="G584" s="3" t="inlineStr">
         <is>
-          <t>Potassium acetate/Sodium acetate anhydrous/Sodium chloride/Dextrose anhydrous/Sodiumphosphatemonobasic monohydrate</t>
+          <t>Potassiumacetate / Sodiumacetateanhydrous / Sodium Chloride / Dextroseanhydrous / Sodiumphosphatemonobasicmonohydrate</t>
         </is>
       </c>
       <c r="H584" s="3" t="inlineStr">
@@ -50847,7 +50847,7 @@
       </c>
       <c r="G585" s="3" t="inlineStr">
         <is>
-          <t>Potassium acetate/Sodium acetate anhydrous/Magnesium chloride Hexahydrate/Sodium chloride/Dextrose anhydrous/Potassiumphosphatemonobasic</t>
+          <t>Potassiumacetate / Sodiumacetateanhydrous / Magnesiumchloride Hexahydrate / Sodium Chloride / Dextroseanhydrous / Potassiumphosphatemonobasic</t>
         </is>
       </c>
       <c r="H585" s="3" t="inlineStr">
@@ -50924,7 +50924,7 @@
       </c>
       <c r="G586" s="3" t="inlineStr">
         <is>
-          <t>LansoprazoleOralDispersible</t>
+          <t>Lansoprazole</t>
         </is>
       </c>
       <c r="H586" s="3" t="inlineStr">
@@ -51102,7 +51102,7 @@
       </c>
       <c r="G588" s="3" t="inlineStr">
         <is>
-          <t>Tamsulosin (HCl) OralDispersible</t>
+          <t>Tamsulosin (HCl)</t>
         </is>
       </c>
       <c r="H588" s="3" t="inlineStr">
@@ -51191,7 +51191,7 @@
       </c>
       <c r="G589" s="3" t="inlineStr">
         <is>
-          <t>Acetylcysteine Granules</t>
+          <t>Acetylcysteine</t>
         </is>
       </c>
       <c r="H589" s="3" t="inlineStr">
@@ -51439,7 +51439,7 @@
       </c>
       <c r="G592" s="3" t="inlineStr">
         <is>
-          <t>Testosterone cypionate</t>
+          <t>Testosteronecypionate</t>
         </is>
       </c>
       <c r="H592" s="3" t="inlineStr">
@@ -51524,7 +51524,7 @@
       </c>
       <c r="G593" s="3" t="inlineStr">
         <is>
-          <t>Tetracycline (HCl) Oph.Oint.</t>
+          <t>Tetracycline (HCl) Oph..</t>
         </is>
       </c>
       <c r="H593" s="3" t="inlineStr">
@@ -52014,7 +52014,7 @@
       </c>
       <c r="G599" s="3" t="inlineStr">
         <is>
-          <t>Timolol (maleate) Oph.Sol'n</t>
+          <t>Timolol (maleate) Oph.</t>
         </is>
       </c>
       <c r="H599" s="3" t="inlineStr">
@@ -52278,7 +52278,7 @@
       </c>
       <c r="G602" s="3" t="inlineStr">
         <is>
-          <t>Pitavastatin/Ezetimibe</t>
+          <t>Pitavastatin / Ezetimibe</t>
         </is>
       </c>
       <c r="H602" s="3" t="inlineStr">
@@ -52367,7 +52367,7 @@
       </c>
       <c r="G603" s="3" t="inlineStr">
         <is>
-          <t>Piroxicam Gel</t>
+          <t>Piroxicam</t>
         </is>
       </c>
       <c r="H603" s="3" t="inlineStr">
@@ -52456,7 +52456,7 @@
       </c>
       <c r="G604" s="3" t="inlineStr">
         <is>
-          <t>InsulinGlargine</t>
+          <t>Insulin Glargine</t>
         </is>
       </c>
       <c r="H604" s="3" t="inlineStr">
@@ -52545,7 +52545,7 @@
       </c>
       <c r="G605" s="3" t="inlineStr">
         <is>
-          <t>Tramadol (HCl)/Acetaminophen</t>
+          <t>Tramadol (HCl) / Acetaminophen</t>
         </is>
       </c>
       <c r="H605" s="3" t="inlineStr">
@@ -52728,7 +52728,7 @@
       </c>
       <c r="G607" s="3" t="inlineStr">
         <is>
-          <t>Tranexamic acid</t>
+          <t>Tranexamic Acid</t>
         </is>
       </c>
       <c r="H607" s="3" t="inlineStr">
@@ -52813,7 +52813,7 @@
       </c>
       <c r="G608" s="3" t="inlineStr">
         <is>
-          <t>Tranexamic acid</t>
+          <t>Tranexamic Acid</t>
         </is>
       </c>
       <c r="H608" s="3" t="inlineStr">
@@ -52983,7 +52983,7 @@
       </c>
       <c r="G610" s="3" t="inlineStr">
         <is>
-          <t>Fluticasonefuroate/Umeclidinium bromide/Vilanteroltrifenatate</t>
+          <t>Fluticasonefuroate / Umeclidiniumbromide / Vilanterol Trifenatate</t>
         </is>
       </c>
       <c r="H610" s="3" t="inlineStr">
@@ -53072,7 +53072,7 @@
       </c>
       <c r="G611" s="3" t="inlineStr">
         <is>
-          <t>Fluticasone/Umeclidinium/VilanterolInhalation Powder</t>
+          <t>Fluticasone / Umeclidinium / Vilanterol Inhalation</t>
         </is>
       </c>
       <c r="H611" s="3" t="inlineStr">
@@ -53161,7 +53161,7 @@
       </c>
       <c r="G612" s="3" t="inlineStr">
         <is>
-          <t>InsulinDegludec</t>
+          <t>Insulin Degludec</t>
         </is>
       </c>
       <c r="H612" s="3" t="inlineStr">
@@ -53256,7 +53256,7 @@
       </c>
       <c r="G613" s="3" t="inlineStr">
         <is>
-          <t>TriamcinoloneacetonideSusp.</t>
+          <t>Triamcinolone Acetonide</t>
         </is>
       </c>
       <c r="H613" s="3" t="inlineStr">
@@ -53341,7 +53341,7 @@
       </c>
       <c r="G614" s="3" t="inlineStr">
         <is>
-          <t>TriamcinoloneacetonideSusp.</t>
+          <t>Triamcinolone Acetonide</t>
         </is>
       </c>
       <c r="H614" s="3" t="inlineStr">
@@ -53594,7 +53594,7 @@
       </c>
       <c r="G617" s="3" t="inlineStr">
         <is>
-          <t>Beclomethasone dipropionate/Formoterol fumarate (dihydrate)/Glycopyrronium (bromide)</t>
+          <t>Beclomethasonedipropionate / Formoterolfumarate (dihydrate) / Glycopyrronium (bromide)</t>
         </is>
       </c>
       <c r="H617" s="3" t="inlineStr">
@@ -53683,7 +53683,7 @@
       </c>
       <c r="G618" s="3" t="inlineStr">
         <is>
-          <t>Triamcinoloneacetonide Nasal Spray</t>
+          <t>Triamcinoloneacetonide</t>
         </is>
       </c>
       <c r="H618" s="3" t="inlineStr">
@@ -53764,7 +53764,7 @@
       </c>
       <c r="G619" s="3" t="inlineStr">
         <is>
-          <t>Abacavir (sulfate)/Dolutegravir (sodium)/Lamivudine</t>
+          <t>Abacavir (sulfate) / Dolutegravir (sodium) / Lamivudine</t>
         </is>
       </c>
       <c r="H619" s="3" t="inlineStr">
@@ -53946,7 +53946,7 @@
       </c>
       <c r="G621" s="3" t="inlineStr">
         <is>
-          <t>Tenofovirdisoproxil (fumarate)/Emtricitabine</t>
+          <t>Tenofovir Disoproxil (fumarate) / Emtricitabine</t>
         </is>
       </c>
       <c r="H621" s="3" t="inlineStr">
@@ -54035,7 +54035,7 @@
       </c>
       <c r="G622" s="3" t="inlineStr">
         <is>
-          <t>Atorvastatin calcium</t>
+          <t>Atorvastatincalcium</t>
         </is>
       </c>
       <c r="H622" s="3" t="inlineStr">
@@ -54124,7 +54124,7 @@
       </c>
       <c r="G623" s="3" t="inlineStr">
         <is>
-          <t>Urea Cream</t>
+          <t>Urea</t>
         </is>
       </c>
       <c r="H623" s="3" t="inlineStr">
@@ -54290,7 +54290,7 @@
       </c>
       <c r="G625" s="3" t="inlineStr">
         <is>
-          <t>Tegafur/Uracil</t>
+          <t>Tegafur / Uracil</t>
         </is>
       </c>
       <c r="H625" s="3" t="inlineStr">
@@ -54551,7 +54551,7 @@
       </c>
       <c r="G628" s="3" t="inlineStr">
         <is>
-          <t>TolterodineL-tartrate</t>
+          <t>Tolterodine L-tartrate</t>
         </is>
       </c>
       <c r="H628" s="3" t="inlineStr">
@@ -54895,7 +54895,7 @@
       </c>
       <c r="G632" s="3" t="inlineStr">
         <is>
-          <t>Ursodeoxycholic acid</t>
+          <t>Ursodeoxycholic Acid</t>
         </is>
       </c>
       <c r="H632" s="3" t="inlineStr">
@@ -55069,7 +55069,7 @@
       </c>
       <c r="G634" s="3" t="inlineStr">
         <is>
-          <t>Progesteronemicronized</t>
+          <t>Progesterone (Micronized)</t>
         </is>
       </c>
       <c r="H634" s="3" t="inlineStr">
@@ -55248,7 +55248,7 @@
       </c>
       <c r="G636" s="3" t="inlineStr">
         <is>
-          <t>Neostigminemethyl sulfate</t>
+          <t>Neostigminemethylsulfate</t>
         </is>
       </c>
       <c r="H636" s="3" t="inlineStr">
@@ -55333,7 +55333,7 @@
       </c>
       <c r="G637" s="3" t="inlineStr">
         <is>
-          <t>Valproate sodium/Valproic acid (equivalenttosodiumvalproate)</t>
+          <t>Valproatesodium / Valproic Acid (equivalenttosodiumvalproate)</t>
         </is>
       </c>
       <c r="H637" s="3" t="inlineStr">
@@ -55737,7 +55737,7 @@
       </c>
       <c r="G642" s="3" t="inlineStr">
         <is>
-          <t>Tenofoviralafenamide fumarate</t>
+          <t>Tenofoviralafenamidefumarate</t>
         </is>
       </c>
       <c r="H642" s="3" t="inlineStr">
@@ -55911,7 +55911,7 @@
       </c>
       <c r="G644" s="3" t="inlineStr">
         <is>
-          <t>Sildenafil citrate</t>
+          <t>Sildenafilcitrate</t>
         </is>
       </c>
       <c r="H644" s="3" t="inlineStr">
@@ -56166,7 +56166,7 @@
       </c>
       <c r="G647" s="3" t="inlineStr">
         <is>
-          <t>Calcium chloride/Glucose</t>
+          <t>Calcium Chloride / Glucose</t>
         </is>
       </c>
       <c r="H647" s="3" t="inlineStr">
@@ -56695,7 +56695,7 @@
       </c>
       <c r="G653" s="3" t="inlineStr">
         <is>
-          <t>Sofosbuvir/Velpatasvir/Voxilaprevir</t>
+          <t>Sofosbuvir / Velpatasvir / Voxilaprevir</t>
         </is>
       </c>
       <c r="H653" s="3" t="inlineStr">
@@ -56871,7 +56871,7 @@
       </c>
       <c r="G655" s="3" t="inlineStr">
         <is>
-          <t>Water for injection</t>
+          <t>Waterforinjection</t>
         </is>
       </c>
       <c r="H655" s="3" t="inlineStr">
@@ -57025,7 +57025,7 @@
       </c>
       <c r="G657" s="3" t="inlineStr">
         <is>
-          <t>Atracurium besylate-Cis (Cisatracurium besylate)</t>
+          <t>Atracuriumbesylate-Cis (Cisatracuriumbesylate)</t>
         </is>
       </c>
       <c r="H657" s="3" t="inlineStr">
@@ -57114,7 +57114,7 @@
       </c>
       <c r="G658" s="3" t="inlineStr">
         <is>
-          <t>Miconazolenitrate Cream</t>
+          <t>Miconazolenitrate</t>
         </is>
       </c>
       <c r="H658" s="3" t="inlineStr">
@@ -57634,7 +57634,7 @@
       </c>
       <c r="G664" s="3" t="inlineStr">
         <is>
-          <t>Dapagliflozin (propanediol)/Metformin (HCl)</t>
+          <t>Dapagliflozin (propanediol) / Metformin (HCl)</t>
         </is>
       </c>
       <c r="H664" s="3" t="inlineStr">
@@ -58072,7 +58072,7 @@
       </c>
       <c r="G669" s="3" t="inlineStr">
         <is>
-          <t>LidocainePump Spray</t>
+          <t>Lidocaine Pump Spray</t>
         </is>
       </c>
       <c r="H669" s="3" t="inlineStr">
@@ -58309,7 +58309,7 @@
       </c>
       <c r="G672" s="3" t="inlineStr">
         <is>
-          <t>Ceftazidime/Avibactam</t>
+          <t>Ceftazidime / Avibactam</t>
         </is>
       </c>
       <c r="H672" s="3" t="inlineStr">
@@ -58402,7 +58402,7 @@
       </c>
       <c r="G673" s="3" t="inlineStr">
         <is>
-          <t>ZincoxideOint.</t>
+          <t>Zincoxide .</t>
         </is>
       </c>
       <c r="H673" s="3" t="inlineStr">
@@ -59021,7 +59021,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G680" s="3" t="inlineStr"/>
+      <c r="G680" s="3" t="inlineStr">
+        <is>
+          <t>Bismuth Subcitrate</t>
+        </is>
+      </c>
       <c r="H680" s="3" t="inlineStr"/>
       <c r="I680" s="2" t="inlineStr">
         <is>
@@ -59100,7 +59104,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G681" s="3" t="inlineStr"/>
+      <c r="G681" s="3" t="inlineStr">
+        <is>
+          <t>Chlorhexidine Gluconate</t>
+        </is>
+      </c>
       <c r="H681" s="3" t="inlineStr"/>
       <c r="I681" s="2" t="inlineStr"/>
       <c r="J681" s="5" t="inlineStr"/>
@@ -59175,7 +59183,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G682" s="3" t="inlineStr"/>
+      <c r="G682" s="3" t="inlineStr">
+        <is>
+          <t>Perflubutane</t>
+        </is>
+      </c>
       <c r="H682" s="3" t="inlineStr"/>
       <c r="I682" s="2" t="inlineStr"/>
       <c r="J682" s="5" t="inlineStr"/>
@@ -59250,7 +59262,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G683" s="3" t="inlineStr"/>
+      <c r="G683" s="3" t="inlineStr">
+        <is>
+          <t>Nicotine</t>
+        </is>
+      </c>
       <c r="H683" s="3" t="inlineStr"/>
       <c r="I683" s="2" t="inlineStr"/>
       <c r="J683" s="5" t="inlineStr"/>
@@ -59394,7 +59410,7 @@
       </c>
       <c r="G685" s="3" t="inlineStr">
         <is>
-          <t>(20meq/100ml/Btl)</t>
+          <t>(20meq / 100ml / Btl)</t>
         </is>
       </c>
       <c r="H685" s="3" t="inlineStr">
@@ -59532,7 +59548,7 @@
       </c>
       <c r="G687" s="3" t="inlineStr">
         <is>
-          <t>Policresulen Sol'n</t>
+          <t>Policresulen</t>
         </is>
       </c>
       <c r="H687" s="3" t="inlineStr">
@@ -59601,7 +59617,7 @@
       </c>
       <c r="G688" s="3" t="inlineStr">
         <is>
-          <t>Proparacaine HCl Eye Sol'n</t>
+          <t>Proparacaine HCl Eye</t>
         </is>
       </c>
       <c r="H688" s="3" t="inlineStr">
@@ -59845,7 +59861,7 @@
       </c>
       <c r="G691" s="3" t="inlineStr">
         <is>
-          <t>Aspirin</t>
+          <t>Aspirin (Acetylsalicylic Acid)</t>
         </is>
       </c>
       <c r="H691" s="3" t="inlineStr">
@@ -60193,7 +60209,7 @@
       </c>
       <c r="G695" s="3" t="inlineStr">
         <is>
-          <t>Biperiden inj. 5mg/ml 1ml</t>
+          <t>Biperiden inj. 5mg / ml 1ml</t>
         </is>
       </c>
       <c r="H695" s="3" t="inlineStr">
@@ -61241,7 +61257,7 @@
       </c>
       <c r="G708" s="3" t="inlineStr">
         <is>
-          <t>M.M.R II (Measles,Mumps,Rubella virus vaccine,live)</t>
+          <t>M.M.R II (Measles / Mumps / Rubella virus vaccine / live)</t>
         </is>
       </c>
       <c r="H708" s="3" t="inlineStr">
@@ -61666,7 +61682,7 @@
       </c>
       <c r="G713" s="3" t="inlineStr">
         <is>
-          <t>Sodium chloride for Irrigation Sol'n</t>
+          <t>Sodium chloride for Irrigation</t>
         </is>
       </c>
       <c r="H713" s="3" t="inlineStr">
@@ -61735,7 +61751,7 @@
       </c>
       <c r="G714" s="3" t="inlineStr">
         <is>
-          <t>Naloxone HCL inj. 0.4mg/ml,1ml</t>
+          <t>Naloxone HCL inj. 0.4mg / ml / 1ml</t>
         </is>
       </c>
       <c r="H714" s="3" t="inlineStr">
@@ -61824,7 +61840,7 @@
       </c>
       <c r="G715" s="3" t="inlineStr">
         <is>
-          <t>Permethrin 50mg/gm, 5%</t>
+          <t>Permethrin 50mg / gm / 5%</t>
         </is>
       </c>
       <c r="H715" s="3" t="inlineStr">
@@ -62152,7 +62168,7 @@
       </c>
       <c r="G719" s="3" t="inlineStr">
         <is>
-          <t>Mepivacaine HCl 36mg+Adrenaline 18mcg......</t>
+          <t>Mepivacaine HCl 36mg + Adrenaline 18mcg......</t>
         </is>
       </c>
       <c r="H719" s="3" t="inlineStr">
@@ -62316,7 +62332,7 @@
       </c>
       <c r="G721" s="3" t="inlineStr">
         <is>
-          <t>Bacitracin Zinc/Polymyxin B (sulfate)/Neomycin (sulfate) Oint.</t>
+          <t>Bacitracin Zinc / Polymyxin B (sulfate) / Neomycin (sulfate) .</t>
         </is>
       </c>
       <c r="H721" s="3" t="inlineStr">
@@ -62527,7 +62543,7 @@
       </c>
       <c r="G724" s="3" t="inlineStr">
         <is>
-          <t>Human Fibrinogen (Clottable Protein)/Aprotinin/Human Thrombin/Calcium chloride Sol'n for Sealant</t>
+          <t>Human Fibrinogen (Clottable Protein) / Aprotinin / Human Thrombin / Calcium chloride for Sealant</t>
         </is>
       </c>
       <c r="H724" s="3" t="inlineStr">
@@ -62681,7 +62697,7 @@
       </c>
       <c r="G726" s="3" t="inlineStr">
         <is>
-          <t>A/H1N1,A/H3N2,B/Phuket</t>
+          <t>A / H1N1 / A / H3N2 / B / Phuket</t>
         </is>
       </c>
       <c r="H726" s="3" t="inlineStr">
@@ -62922,7 +62938,7 @@
       </c>
       <c r="G729" s="3" t="inlineStr">
         <is>
-          <t>Medical Liquid Oxygen</t>
+          <t>Liquid Medical Oxygen</t>
         </is>
       </c>
       <c r="H729" s="3" t="inlineStr">
@@ -63183,7 +63199,7 @@
       </c>
       <c r="G732" s="3" t="inlineStr">
         <is>
-          <t>CO2</t>
+          <t>Carbon Dioxide</t>
         </is>
       </c>
       <c r="H732" s="3" t="inlineStr">
@@ -63588,7 +63604,7 @@
       </c>
       <c r="G737" s="3" t="inlineStr">
         <is>
-          <t>Pitavastatin/Ezetimibe</t>
+          <t>Atorvastatin Calcium / Ezetimibe</t>
         </is>
       </c>
       <c r="H737" s="3" t="inlineStr">
@@ -63677,7 +63693,7 @@
       </c>
       <c r="G738" s="3" t="inlineStr">
         <is>
-          <t>Linagliptin/Metformin</t>
+          <t>Linagliptin / Metformin HCl</t>
         </is>
       </c>
       <c r="H738" s="3" t="inlineStr">
@@ -63768,7 +63784,11 @@
           <t>-</t>
         </is>
       </c>
-      <c r="G739" s="3" t="inlineStr"/>
+      <c r="G739" s="3" t="inlineStr">
+        <is>
+          <t>Sodium Zirconium Cyclosilicate</t>
+        </is>
+      </c>
       <c r="H739" s="3" t="inlineStr"/>
       <c r="I739" s="2" t="inlineStr"/>
       <c r="J739" s="5" t="inlineStr"/>

</xml_diff>